<commit_message>
transfer dataset into mysql workbench and clean some column name
</commit_message>
<xml_diff>
--- a/population.csv.xlsx
+++ b/population.csv.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\My Project\Indian Population Data Analysis\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A4BD8FB3-6457-447E-BB0F-5D7F160F7A4A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DA8B4099-5B02-420F-93F1-66877240B4F4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{FB82829B-6F12-444B-8421-B58D62F0B729}"/>
   </bookViews>
@@ -19,8 +19,8 @@
   </sheets>
   <calcPr calcId="191029"/>
   <pivotCaches>
-    <pivotCache cacheId="5" r:id="rId4"/>
-    <pivotCache cacheId="22" r:id="rId5"/>
+    <pivotCache cacheId="0" r:id="rId4"/>
+    <pivotCache cacheId="1" r:id="rId5"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
   <metadataTypes count="1">
     <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
   </metadataTypes>
@@ -871,7 +871,7 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="33" borderId="10" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="34" borderId="10" xfId="0" applyFill="1" applyBorder="1"/>
@@ -880,20 +880,19 @@
     <xf numFmtId="9" fontId="0" fillId="34" borderId="10" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="35" borderId="10" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="16" fillId="36" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" pivotButton="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="16" fillId="36" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" pivotButton="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" indent="1"/>
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="42">
@@ -2723,7 +2722,191 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{9F7B912B-B7BC-4364-BBA6-38B4B0148DFC}" name="PivotTable4" cacheId="22" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{80C3E7D3-975D-432E-ACA4-EC6B906FDDBE}" name="PivotTable1" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+  <location ref="A5:B12" firstHeaderRow="1" firstDataRow="1" firstDataCol="1" rowPageCount="1" colPageCount="1"/>
+  <pivotFields count="14">
+    <pivotField showAll="0"/>
+    <pivotField axis="axisRow" showAll="0">
+      <items count="37">
+        <item x="31"/>
+        <item x="4"/>
+        <item x="26"/>
+        <item x="13"/>
+        <item x="2"/>
+        <item x="29"/>
+        <item x="15"/>
+        <item x="32"/>
+        <item x="33"/>
+        <item x="17"/>
+        <item x="25"/>
+        <item x="9"/>
+        <item x="16"/>
+        <item x="20"/>
+        <item x="18"/>
+        <item x="12"/>
+        <item x="8"/>
+        <item x="11"/>
+        <item x="34"/>
+        <item x="5"/>
+        <item x="1"/>
+        <item x="23"/>
+        <item x="22"/>
+        <item x="28"/>
+        <item x="24"/>
+        <item x="10"/>
+        <item x="27"/>
+        <item x="14"/>
+        <item x="7"/>
+        <item x="30"/>
+        <item x="6"/>
+        <item x="21"/>
+        <item x="0"/>
+        <item x="19"/>
+        <item x="3"/>
+        <item x="35"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0">
+      <items count="35">
+        <item x="31"/>
+        <item x="30"/>
+        <item x="27"/>
+        <item x="17"/>
+        <item x="29"/>
+        <item x="16"/>
+        <item x="18"/>
+        <item x="28"/>
+        <item x="14"/>
+        <item x="0"/>
+        <item x="2"/>
+        <item x="9"/>
+        <item x="7"/>
+        <item x="1"/>
+        <item x="5"/>
+        <item x="24"/>
+        <item x="32"/>
+        <item x="12"/>
+        <item x="3"/>
+        <item x="13"/>
+        <item x="21"/>
+        <item x="19"/>
+        <item x="20"/>
+        <item x="8"/>
+        <item x="26"/>
+        <item x="10"/>
+        <item x="22"/>
+        <item x="15"/>
+        <item x="23"/>
+        <item x="4"/>
+        <item x="6"/>
+        <item x="25"/>
+        <item x="11"/>
+        <item x="33"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField axis="axisPage" multipleItemSelectionAllowed="1" showAll="0">
+      <items count="37">
+        <item h="1" x="2"/>
+        <item h="1" x="26"/>
+        <item h="1" x="7"/>
+        <item h="1" x="12"/>
+        <item h="1" x="4"/>
+        <item h="1" x="18"/>
+        <item h="1" x="0"/>
+        <item h="1" x="5"/>
+        <item h="1" x="15"/>
+        <item h="1" x="13"/>
+        <item h="1" x="10"/>
+        <item h="1" x="22"/>
+        <item h="1" x="8"/>
+        <item h="1" x="16"/>
+        <item x="14"/>
+        <item x="32"/>
+        <item h="1" x="3"/>
+        <item h="1" x="9"/>
+        <item h="1" x="23"/>
+        <item h="1" x="24"/>
+        <item x="19"/>
+        <item h="1" x="6"/>
+        <item h="1" x="30"/>
+        <item h="1" x="1"/>
+        <item h="1" x="20"/>
+        <item h="1" x="27"/>
+        <item h="1" x="29"/>
+        <item h="1" x="17"/>
+        <item x="31"/>
+        <item h="1" x="33"/>
+        <item h="1" x="21"/>
+        <item h="1" x="25"/>
+        <item h="1" x="28"/>
+        <item x="34"/>
+        <item x="11"/>
+        <item h="1" x="35"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField dataField="1" showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+  </pivotFields>
+  <rowFields count="1">
+    <field x="1"/>
+  </rowFields>
+  <rowItems count="7">
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="7"/>
+    </i>
+    <i>
+      <x v="17"/>
+    </i>
+    <i>
+      <x v="18"/>
+    </i>
+    <i>
+      <x v="27"/>
+    </i>
+    <i>
+      <x v="33"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colItems count="1">
+    <i/>
+  </colItems>
+  <pageFields count="1">
+    <pageField fld="8" hier="-1"/>
+  </pageFields>
+  <dataFields count="1">
+    <dataField name="Sum of Rural Population" fld="9" baseField="0" baseItem="0"/>
+  </dataFields>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
+<file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{9F7B912B-B7BC-4364-BBA6-38B4B0148DFC}" name="PivotTable4" cacheId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="L5:M76" firstHeaderRow="1" firstDataRow="1" firstDataCol="1" rowPageCount="1" colPageCount="1"/>
   <pivotFields count="14">
     <pivotField showAll="0"/>
@@ -3133,8 +3316,8 @@
 </pivotTableDefinition>
 </file>
 
-<file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{51E9E64C-34E6-49FF-ABC4-DCBA46C9B4F0}" name="PivotTable3" cacheId="22" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+<file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{51E9E64C-34E6-49FF-ABC4-DCBA46C9B4F0}" name="PivotTable3" cacheId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="H5:J39" firstHeaderRow="0" firstDataRow="1" firstDataCol="1" rowPageCount="1" colPageCount="1"/>
   <pivotFields count="14">
     <pivotField showAll="0"/>
@@ -3402,8 +3585,8 @@
 </pivotTableDefinition>
 </file>
 
-<file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{283C2D54-EA66-46DD-A52C-DBEC61E2F94E}" name="PivotTable2" cacheId="22" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+<file path=xl/pivotTables/pivotTable4.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{283C2D54-EA66-46DD-A52C-DBEC61E2F94E}" name="PivotTable2" cacheId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
   <location ref="E5:F41" firstHeaderRow="1" firstDataRow="1" firstDataCol="1" rowPageCount="1" colPageCount="1"/>
   <pivotFields count="14">
     <pivotField showAll="0">
@@ -3733,190 +3916,6 @@
   </pageFields>
   <dataFields count="1">
     <dataField name="Sum of Females" fld="6" baseField="0" baseItem="0" numFmtId="3"/>
-  </dataFields>
-  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
-      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
-    </ext>
-    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
-      <xpdl:pivotTableDefinition16/>
-    </ext>
-  </extLst>
-</pivotTableDefinition>
-</file>
-
-<file path=xl/pivotTables/pivotTable4.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{80C3E7D3-975D-432E-ACA4-EC6B906FDDBE}" name="PivotTable1" cacheId="5" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
-  <location ref="A5:B12" firstHeaderRow="1" firstDataRow="1" firstDataCol="1" rowPageCount="1" colPageCount="1"/>
-  <pivotFields count="14">
-    <pivotField showAll="0"/>
-    <pivotField axis="axisRow" showAll="0">
-      <items count="37">
-        <item x="31"/>
-        <item x="4"/>
-        <item x="26"/>
-        <item x="13"/>
-        <item x="2"/>
-        <item x="29"/>
-        <item x="15"/>
-        <item x="32"/>
-        <item x="33"/>
-        <item x="17"/>
-        <item x="25"/>
-        <item x="9"/>
-        <item x="16"/>
-        <item x="20"/>
-        <item x="18"/>
-        <item x="12"/>
-        <item x="8"/>
-        <item x="11"/>
-        <item x="34"/>
-        <item x="5"/>
-        <item x="1"/>
-        <item x="23"/>
-        <item x="22"/>
-        <item x="28"/>
-        <item x="24"/>
-        <item x="10"/>
-        <item x="27"/>
-        <item x="14"/>
-        <item x="7"/>
-        <item x="30"/>
-        <item x="6"/>
-        <item x="21"/>
-        <item x="0"/>
-        <item x="19"/>
-        <item x="3"/>
-        <item x="35"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0">
-      <items count="35">
-        <item x="31"/>
-        <item x="30"/>
-        <item x="27"/>
-        <item x="17"/>
-        <item x="29"/>
-        <item x="16"/>
-        <item x="18"/>
-        <item x="28"/>
-        <item x="14"/>
-        <item x="0"/>
-        <item x="2"/>
-        <item x="9"/>
-        <item x="7"/>
-        <item x="1"/>
-        <item x="5"/>
-        <item x="24"/>
-        <item x="32"/>
-        <item x="12"/>
-        <item x="3"/>
-        <item x="13"/>
-        <item x="21"/>
-        <item x="19"/>
-        <item x="20"/>
-        <item x="8"/>
-        <item x="26"/>
-        <item x="10"/>
-        <item x="22"/>
-        <item x="15"/>
-        <item x="23"/>
-        <item x="4"/>
-        <item x="6"/>
-        <item x="25"/>
-        <item x="11"/>
-        <item x="33"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField axis="axisPage" multipleItemSelectionAllowed="1" showAll="0">
-      <items count="37">
-        <item h="1" x="2"/>
-        <item h="1" x="26"/>
-        <item h="1" x="7"/>
-        <item h="1" x="12"/>
-        <item h="1" x="4"/>
-        <item h="1" x="18"/>
-        <item h="1" x="0"/>
-        <item h="1" x="5"/>
-        <item h="1" x="15"/>
-        <item h="1" x="13"/>
-        <item h="1" x="10"/>
-        <item h="1" x="22"/>
-        <item h="1" x="8"/>
-        <item h="1" x="16"/>
-        <item x="14"/>
-        <item x="32"/>
-        <item h="1" x="3"/>
-        <item h="1" x="9"/>
-        <item h="1" x="23"/>
-        <item h="1" x="24"/>
-        <item x="19"/>
-        <item h="1" x="6"/>
-        <item h="1" x="30"/>
-        <item h="1" x="1"/>
-        <item h="1" x="20"/>
-        <item h="1" x="27"/>
-        <item h="1" x="29"/>
-        <item h="1" x="17"/>
-        <item x="31"/>
-        <item h="1" x="33"/>
-        <item h="1" x="21"/>
-        <item h="1" x="25"/>
-        <item h="1" x="28"/>
-        <item x="34"/>
-        <item x="11"/>
-        <item h="1" x="35"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField dataField="1" showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-  </pivotFields>
-  <rowFields count="1">
-    <field x="1"/>
-  </rowFields>
-  <rowItems count="7">
-    <i>
-      <x/>
-    </i>
-    <i>
-      <x v="7"/>
-    </i>
-    <i>
-      <x v="17"/>
-    </i>
-    <i>
-      <x v="18"/>
-    </i>
-    <i>
-      <x v="27"/>
-    </i>
-    <i>
-      <x v="33"/>
-    </i>
-    <i t="grand">
-      <x/>
-    </i>
-  </rowItems>
-  <colItems count="1">
-    <i/>
-  </colItems>
-  <pageFields count="1">
-    <pageField fld="8" hier="-1"/>
-  </pageFields>
-  <dataFields count="1">
-    <dataField name="Sum of Rural Population" fld="9" baseField="0" baseItem="0"/>
   </dataFields>
   <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
   <extLst>
@@ -4250,20 +4249,20 @@
   <dimension ref="A1:N36"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="5" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="25.109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="17.77734375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="11.6640625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="17.77734375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="11.6640625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="10.6640625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="11.44140625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="14.44140625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="14.21875" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="14.88671875" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="12.109375" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="16" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="17" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="5.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="26.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="18.6640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12.5546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="19.109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.5546875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="11.44140625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="12" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="15" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="15.21875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="16" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="12.5546875" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="17.109375" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="17.88671875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:14" x14ac:dyDescent="0.3">
@@ -5876,19 +5875,19 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="A2" s="9" t="s">
+      <c r="A2" s="12" t="s">
         <v>79</v>
       </c>
-      <c r="B2" s="9"/>
-      <c r="C2" s="9"/>
-      <c r="E2" s="9" t="s">
+      <c r="B2" s="12"/>
+      <c r="C2" s="12"/>
+      <c r="E2" s="12" t="s">
         <v>82</v>
       </c>
-      <c r="F2" s="9"/>
-      <c r="H2" s="9" t="s">
+      <c r="F2" s="12"/>
+      <c r="H2" s="12" t="s">
         <v>85</v>
       </c>
-      <c r="I2" s="9"/>
+      <c r="I2" s="12"/>
       <c r="L2" s="7" t="s">
         <v>1</v>
       </c>
@@ -5930,22 +5929,22 @@
       </c>
     </row>
     <row r="3" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="A3" s="8">
+      <c r="A3" s="13">
         <f>MAX(population!E2:E36)</f>
         <v>16.5</v>
       </c>
-      <c r="B3" s="8"/>
-      <c r="C3" s="8"/>
-      <c r="E3" s="8">
+      <c r="B3" s="13"/>
+      <c r="C3" s="13"/>
+      <c r="E3" s="13">
         <f>MAX(population!H2:H36)</f>
         <v>1084</v>
       </c>
-      <c r="F3" s="8"/>
-      <c r="H3" s="8">
+      <c r="F3" s="13"/>
+      <c r="H3" s="13">
         <f>MAX(population!I2:I36)</f>
         <v>94</v>
       </c>
-      <c r="I3" s="8"/>
+      <c r="I3" s="13"/>
       <c r="L3" s="6" t="s">
         <v>13</v>
       </c>
@@ -6030,19 +6029,19 @@
       </c>
     </row>
     <row r="5" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="A5" s="9" t="s">
+      <c r="A5" s="12" t="s">
         <v>80</v>
       </c>
-      <c r="B5" s="9"/>
-      <c r="C5" s="9"/>
-      <c r="E5" s="9" t="s">
+      <c r="B5" s="12"/>
+      <c r="C5" s="12"/>
+      <c r="E5" s="12" t="s">
         <v>83</v>
       </c>
-      <c r="F5" s="9"/>
-      <c r="H5" s="9" t="s">
+      <c r="F5" s="12"/>
+      <c r="H5" s="12" t="s">
         <v>86</v>
       </c>
-      <c r="I5" s="9"/>
+      <c r="I5" s="12"/>
       <c r="L5" s="6" t="s">
         <v>54</v>
       </c>
@@ -6085,22 +6084,22 @@
       </c>
     </row>
     <row r="6" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="A6" s="8">
+      <c r="A6" s="13">
         <f>MIN(population!E2:E36)</f>
         <v>0.01</v>
       </c>
-      <c r="B6" s="8"/>
-      <c r="C6" s="8"/>
-      <c r="E6" s="8">
+      <c r="B6" s="13"/>
+      <c r="C6" s="13"/>
+      <c r="E6" s="13">
         <f>MIN(population!H2:H36)</f>
         <v>618</v>
       </c>
-      <c r="F6" s="8"/>
-      <c r="H6" s="8">
+      <c r="F6" s="13"/>
+      <c r="H6" s="13">
         <f>MIN(population!I2:I36)</f>
         <v>61.8</v>
       </c>
-      <c r="I6" s="8"/>
+      <c r="I6" s="13"/>
       <c r="L6" s="6" t="s">
         <v>68</v>
       </c>
@@ -6185,19 +6184,19 @@
       </c>
     </row>
     <row r="8" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="A8" s="9" t="s">
+      <c r="A8" s="12" t="s">
         <v>81</v>
       </c>
-      <c r="B8" s="9"/>
-      <c r="C8" s="9"/>
-      <c r="E8" s="9" t="s">
+      <c r="B8" s="12"/>
+      <c r="C8" s="12"/>
+      <c r="E8" s="12" t="s">
         <v>84</v>
       </c>
-      <c r="F8" s="9"/>
-      <c r="H8" s="9" t="s">
+      <c r="F8" s="12"/>
+      <c r="H8" s="12" t="s">
         <v>87</v>
       </c>
-      <c r="I8" s="9"/>
+      <c r="I8" s="12"/>
       <c r="L8" s="6" t="s">
         <v>62</v>
       </c>
@@ -6240,22 +6239,22 @@
       </c>
     </row>
     <row r="9" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="A9" s="8">
+      <c r="A9" s="13">
         <f>AVERAGE(population!E2:E36)</f>
         <v>2.8568571428571428</v>
       </c>
-      <c r="B9" s="8"/>
-      <c r="C9" s="8"/>
-      <c r="E9" s="8">
+      <c r="B9" s="13"/>
+      <c r="C9" s="13"/>
+      <c r="E9" s="13">
         <f>AVERAGE(population!H2:H36)</f>
         <v>931.2285714285714</v>
       </c>
-      <c r="F9" s="8"/>
-      <c r="H9" s="8">
+      <c r="F9" s="13"/>
+      <c r="H9" s="13">
         <f>AVERAGE(population!I11)</f>
         <v>78.03</v>
       </c>
-      <c r="I9" s="8"/>
+      <c r="I9" s="13"/>
       <c r="L9" s="6" t="s">
         <v>66</v>
       </c>
@@ -6299,11 +6298,12 @@
     </row>
   </sheetData>
   <mergeCells count="18">
-    <mergeCell ref="H2:I2"/>
-    <mergeCell ref="H3:I3"/>
-    <mergeCell ref="H5:I5"/>
-    <mergeCell ref="H6:I6"/>
-    <mergeCell ref="H8:I8"/>
+    <mergeCell ref="A9:C9"/>
+    <mergeCell ref="A2:C2"/>
+    <mergeCell ref="A3:C3"/>
+    <mergeCell ref="A5:C5"/>
+    <mergeCell ref="A6:C6"/>
+    <mergeCell ref="A8:C8"/>
     <mergeCell ref="H9:I9"/>
     <mergeCell ref="E2:F2"/>
     <mergeCell ref="E3:F3"/>
@@ -6311,12 +6311,11 @@
     <mergeCell ref="E6:F6"/>
     <mergeCell ref="E8:F8"/>
     <mergeCell ref="E9:F9"/>
-    <mergeCell ref="A2:C2"/>
-    <mergeCell ref="A3:C3"/>
-    <mergeCell ref="A5:C5"/>
-    <mergeCell ref="A6:C6"/>
-    <mergeCell ref="A8:C8"/>
-    <mergeCell ref="A9:C9"/>
+    <mergeCell ref="H2:I2"/>
+    <mergeCell ref="H3:I3"/>
+    <mergeCell ref="H5:I5"/>
+    <mergeCell ref="H6:I6"/>
+    <mergeCell ref="H8:I8"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
@@ -6374,25 +6373,25 @@
   </cols>
   <sheetData>
     <row r="3" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A3" s="10" t="s">
+      <c r="A3" s="8" t="s">
         <v>7</v>
       </c>
       <c r="B3" t="s">
         <v>92</v>
       </c>
-      <c r="E3" s="10" t="s">
+      <c r="E3" s="8" t="s">
         <v>78</v>
       </c>
       <c r="F3" t="s">
         <v>91</v>
       </c>
-      <c r="H3" s="10" t="s">
+      <c r="H3" s="8" t="s">
         <v>4</v>
       </c>
       <c r="I3" t="s">
         <v>91</v>
       </c>
-      <c r="L3" s="10" t="s">
+      <c r="L3" s="8" t="s">
         <v>10</v>
       </c>
       <c r="M3" t="s">
@@ -6400,19 +6399,19 @@
       </c>
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A5" s="10" t="s">
+      <c r="A5" s="8" t="s">
         <v>88</v>
       </c>
       <c r="B5" t="s">
         <v>90</v>
       </c>
-      <c r="E5" s="10" t="s">
+      <c r="E5" s="8" t="s">
         <v>88</v>
       </c>
       <c r="F5" t="s">
         <v>93</v>
       </c>
-      <c r="H5" s="10" t="s">
+      <c r="H5" s="8" t="s">
         <v>88</v>
       </c>
       <c r="I5" t="s">
@@ -6421,7 +6420,7 @@
       <c r="J5" t="s">
         <v>90</v>
       </c>
-      <c r="L5" s="10" t="s">
+      <c r="L5" s="8" t="s">
         <v>88</v>
       </c>
       <c r="M5" t="s">
@@ -6429,1134 +6428,1134 @@
       </c>
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A6" s="11" t="s">
+      <c r="A6" s="9" t="s">
         <v>70</v>
       </c>
-      <c r="B6" s="12">
+      <c r="B6">
         <v>244411</v>
       </c>
-      <c r="E6" s="11" t="s">
+      <c r="E6" s="9" t="s">
         <v>70</v>
       </c>
-      <c r="F6" s="13">
+      <c r="F6" s="10">
         <v>177710</v>
       </c>
-      <c r="H6" s="11" t="s">
+      <c r="H6" s="9" t="s">
         <v>53</v>
       </c>
-      <c r="I6" s="13">
+      <c r="I6" s="10">
         <v>960981</v>
       </c>
-      <c r="J6" s="13">
+      <c r="J6" s="10">
         <v>2710051</v>
       </c>
-      <c r="L6" s="11" t="s">
+      <c r="L6" s="9" t="s">
         <v>70</v>
       </c>
-      <c r="M6" s="12">
+      <c r="M6">
         <v>0.03</v>
       </c>
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A7" s="11" t="s">
+      <c r="A7" s="9" t="s">
         <v>72</v>
       </c>
-      <c r="B7" s="12">
+      <c r="B7">
         <v>183024</v>
       </c>
-      <c r="E7" s="11" t="s">
+      <c r="E7" s="9" t="s">
         <v>21</v>
       </c>
-      <c r="F7" s="13">
+      <c r="F7" s="10">
         <v>42138631</v>
       </c>
-      <c r="H7" s="11" t="s">
+      <c r="H7" s="9" t="s">
         <v>67</v>
       </c>
-      <c r="I7" s="13">
+      <c r="I7" s="10">
         <v>561997</v>
       </c>
-      <c r="J7" s="13">
+      <c r="J7" s="10">
         <v>529037</v>
       </c>
-      <c r="L7" s="14" t="s">
+      <c r="L7" s="11" t="s">
         <v>71</v>
       </c>
-      <c r="M7" s="12">
+      <c r="M7">
         <v>0.03</v>
       </c>
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A8" s="11" t="s">
+      <c r="A8" s="9" t="s">
         <v>35</v>
       </c>
-      <c r="B8" s="12">
+      <c r="B8">
         <v>17445506</v>
       </c>
-      <c r="E8" s="11" t="s">
+      <c r="E8" s="9" t="s">
         <v>62</v>
       </c>
-      <c r="F8" s="13">
+      <c r="F8" s="10">
         <v>669815</v>
       </c>
-      <c r="H8" s="11" t="s">
+      <c r="H8" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="I8" s="13">
+      <c r="I8" s="10">
         <v>23578175</v>
       </c>
-      <c r="J8" s="13">
+      <c r="J8" s="10">
         <v>37552529</v>
       </c>
-      <c r="L8" s="11" t="s">
+      <c r="L8" s="9" t="s">
         <v>21</v>
       </c>
-      <c r="M8" s="12">
+      <c r="M8">
         <v>6.99</v>
       </c>
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A9" s="11" t="s">
+      <c r="A9" s="9" t="s">
         <v>76</v>
       </c>
-      <c r="B9" s="12">
+      <c r="B9">
         <v>14121</v>
       </c>
-      <c r="E9" s="11" t="s">
+      <c r="E9" s="9" t="s">
         <v>39</v>
       </c>
-      <c r="F9" s="13">
+      <c r="F9" s="10">
         <v>15266133</v>
       </c>
-      <c r="H9" s="11" t="s">
+      <c r="H9" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="I9" s="13">
+      <c r="I9" s="10">
         <v>20059666</v>
       </c>
-      <c r="J9" s="13">
+      <c r="J9" s="10">
         <v>52537899</v>
       </c>
-      <c r="L9" s="14" t="s">
+      <c r="L9" s="11" t="s">
         <v>22</v>
       </c>
-      <c r="M9" s="12">
+      <c r="M9">
         <v>6.99</v>
       </c>
     </row>
     <row r="10" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A10" s="11" t="s">
+      <c r="A10" s="9" t="s">
         <v>41</v>
       </c>
-      <c r="B10" s="12">
+      <c r="B10">
         <v>17316800</v>
       </c>
-      <c r="E10" s="11" t="s">
+      <c r="E10" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="F10" s="13">
+      <c r="F10" s="10">
         <v>49821295</v>
       </c>
-      <c r="H10" s="11" t="s">
+      <c r="H10" s="9" t="s">
         <v>34</v>
       </c>
-      <c r="I10" s="13">
+      <c r="I10" s="10">
         <v>6996124</v>
       </c>
-      <c r="J10" s="13">
+      <c r="J10" s="10">
         <v>34951234</v>
       </c>
-      <c r="L10" s="11" t="s">
+      <c r="L10" s="9" t="s">
         <v>62</v>
       </c>
-      <c r="M10" s="12">
+      <c r="M10">
         <v>0.11</v>
       </c>
     </row>
     <row r="11" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A11" s="11" t="s">
+      <c r="A11" s="9" t="s">
         <v>48</v>
       </c>
-      <c r="B11" s="12">
+      <c r="B11">
         <v>7025583</v>
       </c>
-      <c r="E11" s="11" t="s">
+      <c r="E11" s="9" t="s">
         <v>42</v>
       </c>
-      <c r="F11" s="13">
+      <c r="F11" s="10">
         <v>474787</v>
       </c>
-      <c r="H11" s="11" t="s">
+      <c r="H11" s="9" t="s">
         <v>42</v>
       </c>
-      <c r="I11" s="13">
+      <c r="I11" s="10">
         <v>20234706</v>
       </c>
-      <c r="J11" s="13">
+      <c r="J11" s="10">
         <v>33877297</v>
       </c>
-      <c r="L11" s="14" t="s">
+      <c r="L11" s="11" t="s">
         <v>63</v>
       </c>
-      <c r="M11" s="12">
+      <c r="M11">
         <v>0.11</v>
       </c>
     </row>
     <row r="12" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A12" s="11" t="s">
+      <c r="A12" s="9" t="s">
         <v>89</v>
       </c>
-      <c r="B12" s="12">
+      <c r="B12">
         <v>42229445</v>
       </c>
-      <c r="E12" s="11" t="s">
+      <c r="E12" s="9" t="s">
         <v>43</v>
       </c>
-      <c r="F12" s="13">
+      <c r="F12" s="10">
         <v>12712303</v>
       </c>
-      <c r="H12" s="11" t="s">
+      <c r="H12" s="9" t="s">
         <v>26</v>
       </c>
-      <c r="I12" s="13">
+      <c r="I12" s="10">
         <v>34949729</v>
       </c>
-      <c r="J12" s="13">
+      <c r="J12" s="10">
         <v>37189229</v>
       </c>
-      <c r="L12" s="11" t="s">
+      <c r="L12" s="9" t="s">
         <v>39</v>
       </c>
-      <c r="M12" s="12">
+      <c r="M12">
         <v>2.58</v>
       </c>
     </row>
     <row r="13" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="E13" s="11" t="s">
+      <c r="E13" s="9" t="s">
         <v>72</v>
       </c>
-      <c r="F13" s="13">
+      <c r="F13" s="10">
         <v>149949</v>
       </c>
-      <c r="H13" s="11" t="s">
+      <c r="H13" s="9" t="s">
         <v>75</v>
       </c>
-      <c r="I13" s="13">
+      <c r="I13" s="10">
         <v>182580</v>
       </c>
-      <c r="J13" s="13">
+      <c r="J13" s="10">
         <v>60331</v>
       </c>
-      <c r="L13" s="14" t="s">
+      <c r="L13" s="11" t="s">
         <v>40</v>
       </c>
-      <c r="M13" s="12">
+      <c r="M13">
         <v>2.58</v>
       </c>
     </row>
     <row r="14" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="E14" s="11" t="s">
+      <c r="E14" s="9" t="s">
         <v>74</v>
       </c>
-      <c r="F14" s="13">
+      <c r="F14" s="10">
         <v>92946</v>
       </c>
-      <c r="H14" s="11" t="s">
+      <c r="H14" s="9" t="s">
         <v>49</v>
       </c>
-      <c r="I14" s="13">
+      <c r="I14" s="10">
         <v>3091169</v>
       </c>
-      <c r="J14" s="13">
+      <c r="J14" s="10">
         <v>7025583</v>
       </c>
-      <c r="L14" s="11" t="s">
+      <c r="L14" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="M14" s="12">
+      <c r="M14">
         <v>8.6</v>
       </c>
     </row>
     <row r="15" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="E15" s="11" t="s">
+      <c r="E15" s="9" t="s">
         <v>46</v>
       </c>
-      <c r="F15" s="13">
+      <c r="F15" s="10">
         <v>7800615</v>
       </c>
-      <c r="H15" s="11" t="s">
+      <c r="H15" s="9" t="s">
         <v>46</v>
       </c>
-      <c r="I15" s="13">
+      <c r="I15" s="10">
         <v>12905780</v>
       </c>
-      <c r="J15" s="13">
+      <c r="J15" s="10">
         <v>944727</v>
       </c>
-      <c r="L15" s="14" t="s">
+      <c r="L15" s="11" t="s">
         <v>18</v>
       </c>
-      <c r="M15" s="12">
+      <c r="M15">
         <v>8.6</v>
       </c>
     </row>
     <row r="16" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="E16" s="11" t="s">
+      <c r="E16" s="9" t="s">
         <v>60</v>
       </c>
-      <c r="F16" s="13">
+      <c r="F16" s="10">
         <v>719405</v>
       </c>
-      <c r="H16" s="11" t="s">
+      <c r="H16" s="9" t="s">
         <v>40</v>
       </c>
-      <c r="I16" s="13">
+      <c r="I16" s="10">
         <v>4388756</v>
       </c>
-      <c r="J16" s="13">
+      <c r="J16" s="10">
         <v>26780526</v>
       </c>
-      <c r="L16" s="11" t="s">
+      <c r="L16" s="9" t="s">
         <v>42</v>
       </c>
-      <c r="M16" s="12">
+      <c r="M16">
         <v>0.09</v>
       </c>
     </row>
     <row r="17" spans="5:13" x14ac:dyDescent="0.3">
-      <c r="E17" s="11" t="s">
+      <c r="E17" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="F17" s="13">
+      <c r="F17" s="10">
         <v>28948432</v>
       </c>
-      <c r="H17" s="11" t="s">
+      <c r="H17" s="9" t="s">
         <v>32</v>
       </c>
-      <c r="I17" s="13">
+      <c r="I17" s="10">
         <v>25712811</v>
       </c>
-      <c r="J17" s="13">
+      <c r="J17" s="10">
         <v>34670817</v>
       </c>
-      <c r="L17" s="14" t="s">
+      <c r="L17" s="11" t="s">
         <v>42</v>
       </c>
-      <c r="M17" s="12">
+      <c r="M17">
         <v>0.09</v>
       </c>
     </row>
     <row r="18" spans="5:13" x14ac:dyDescent="0.3">
-      <c r="E18" s="11" t="s">
+      <c r="E18" s="9" t="s">
         <v>45</v>
       </c>
-      <c r="F18" s="13">
+      <c r="F18" s="10">
         <v>11856728</v>
       </c>
-      <c r="H18" s="11" t="s">
+      <c r="H18" s="9" t="s">
         <v>69</v>
       </c>
-      <c r="I18" s="13">
+      <c r="I18" s="10">
         <v>151726</v>
       </c>
-      <c r="J18" s="13">
+      <c r="J18" s="10">
         <v>455962</v>
       </c>
-      <c r="L18" s="11" t="s">
+      <c r="L18" s="9" t="s">
         <v>43</v>
       </c>
-      <c r="M18" s="12">
+      <c r="M18">
         <v>2.11</v>
       </c>
     </row>
     <row r="19" spans="5:13" x14ac:dyDescent="0.3">
-      <c r="E19" s="11" t="s">
+      <c r="E19" s="9" t="s">
         <v>50</v>
       </c>
-      <c r="F19" s="13">
+      <c r="F19" s="10">
         <v>3382729</v>
       </c>
-      <c r="H19" s="11" t="s">
+      <c r="H19" s="9" t="s">
         <v>22</v>
       </c>
-      <c r="I19" s="13">
+      <c r="I19" s="10">
         <v>28219075</v>
       </c>
-      <c r="J19" s="13">
+      <c r="J19" s="10">
         <v>56361702</v>
       </c>
-      <c r="L19" s="14" t="s">
+      <c r="L19" s="11" t="s">
         <v>44</v>
       </c>
-      <c r="M19" s="12">
+      <c r="M19">
         <v>2.11</v>
       </c>
     </row>
     <row r="20" spans="5:13" x14ac:dyDescent="0.3">
-      <c r="E20" s="11" t="s">
+      <c r="E20" s="9" t="s">
         <v>47</v>
       </c>
-      <c r="F20" s="13">
+      <c r="F20" s="10">
         <v>5900640</v>
       </c>
-      <c r="H20" s="11" t="s">
+      <c r="H20" s="9" t="s">
         <v>57</v>
       </c>
-      <c r="I20" s="13">
+      <c r="I20" s="10">
         <v>822132</v>
       </c>
-      <c r="J20" s="13">
+      <c r="J20" s="10">
         <v>1899624</v>
       </c>
-      <c r="L20" s="11" t="s">
+      <c r="L20" s="9" t="s">
         <v>72</v>
       </c>
-      <c r="M20" s="12">
+      <c r="M20">
         <v>0.03</v>
       </c>
     </row>
     <row r="21" spans="5:13" x14ac:dyDescent="0.3">
-      <c r="E21" s="11" t="s">
+      <c r="E21" s="9" t="s">
         <v>37</v>
       </c>
-      <c r="F21" s="13">
+      <c r="F21" s="10">
         <v>16057819</v>
       </c>
-      <c r="H21" s="11" t="s">
+      <c r="H21" s="9" t="s">
         <v>63</v>
       </c>
-      <c r="I21" s="13">
+      <c r="I21" s="10">
         <v>313446</v>
       </c>
-      <c r="J21" s="13">
+      <c r="J21" s="10">
         <v>1069165</v>
       </c>
-      <c r="L21" s="14" t="s">
+      <c r="L21" s="11" t="s">
         <v>73</v>
       </c>
-      <c r="M21" s="12">
+      <c r="M21">
         <v>0.03</v>
       </c>
     </row>
     <row r="22" spans="5:13" x14ac:dyDescent="0.3">
-      <c r="E22" s="11" t="s">
+      <c r="E22" s="9" t="s">
         <v>29</v>
       </c>
-      <c r="F22" s="13">
+      <c r="F22" s="10">
         <v>30128640</v>
       </c>
-      <c r="H22" s="11" t="s">
+      <c r="H22" s="9" t="s">
         <v>28</v>
       </c>
-      <c r="I22" s="13">
+      <c r="I22" s="10">
         <v>17080776</v>
       </c>
-      <c r="J22" s="13">
+      <c r="J22" s="10">
         <v>51540236</v>
       </c>
-      <c r="L22" s="11" t="s">
+      <c r="L22" s="9" t="s">
         <v>74</v>
       </c>
-      <c r="M22" s="12">
+      <c r="M22">
         <v>0.02</v>
       </c>
     </row>
     <row r="23" spans="5:13" x14ac:dyDescent="0.3">
-      <c r="E23" s="11" t="s">
+      <c r="E23" s="9" t="s">
         <v>35</v>
       </c>
-      <c r="F23" s="13">
+      <c r="F23" s="10">
         <v>17378649</v>
       </c>
-      <c r="H23" s="11" t="s">
+      <c r="H23" s="9" t="s">
         <v>47</v>
       </c>
-      <c r="I23" s="13">
+      <c r="I23" s="10">
         <v>3414106</v>
       </c>
-      <c r="J23" s="13">
+      <c r="J23" s="10">
         <v>9134820</v>
       </c>
-      <c r="L23" s="14" t="s">
+      <c r="L23" s="11" t="s">
         <v>75</v>
       </c>
-      <c r="M23" s="12">
+      <c r="M23">
         <v>0.02</v>
       </c>
     </row>
     <row r="24" spans="5:13" x14ac:dyDescent="0.3">
-      <c r="E24" s="11" t="s">
+      <c r="E24" s="9" t="s">
         <v>76</v>
       </c>
-      <c r="F24" s="13">
+      <c r="F24" s="10">
         <v>31350</v>
       </c>
-      <c r="H24" s="11" t="s">
+      <c r="H24" s="9" t="s">
         <v>77</v>
       </c>
-      <c r="I24" s="13">
+      <c r="I24" s="10">
         <v>50308</v>
       </c>
-      <c r="J24" s="13">
+      <c r="J24" s="10">
         <v>14121</v>
       </c>
-      <c r="L24" s="11" t="s">
+      <c r="L24" s="9" t="s">
         <v>46</v>
       </c>
-      <c r="M24" s="12">
+      <c r="M24">
         <v>1.39</v>
       </c>
     </row>
     <row r="25" spans="5:13" x14ac:dyDescent="0.3">
-      <c r="E25" s="11" t="s">
+      <c r="E25" s="9" t="s">
         <v>23</v>
       </c>
-      <c r="F25" s="13">
+      <c r="F25" s="10">
         <v>35014503</v>
       </c>
-      <c r="H25" s="11" t="s">
+      <c r="H25" s="9" t="s">
         <v>59</v>
       </c>
-      <c r="I25" s="13">
+      <c r="I25" s="10">
         <v>573741</v>
       </c>
-      <c r="J25" s="13">
+      <c r="J25" s="10">
         <v>1406861</v>
       </c>
-      <c r="L25" s="14" t="s">
+      <c r="L25" s="11" t="s">
         <v>46</v>
       </c>
-      <c r="M25" s="12">
+      <c r="M25">
         <v>1.39</v>
       </c>
     </row>
     <row r="26" spans="5:13" x14ac:dyDescent="0.3">
-      <c r="E26" s="11" t="s">
+      <c r="E26" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="F26" s="13">
+      <c r="F26" s="10">
         <v>54131277</v>
       </c>
-      <c r="H26" s="11" t="s">
+      <c r="H26" s="9" t="s">
         <v>20</v>
       </c>
-      <c r="I26" s="13">
+      <c r="I26" s="10">
         <v>29134060</v>
       </c>
-      <c r="J26" s="13">
+      <c r="J26" s="10">
         <v>62213676</v>
       </c>
-      <c r="L26" s="11" t="s">
+      <c r="L26" s="9" t="s">
         <v>60</v>
       </c>
-      <c r="M26" s="12">
+      <c r="M26">
         <v>0.12</v>
       </c>
     </row>
     <row r="27" spans="5:13" x14ac:dyDescent="0.3">
-      <c r="E27" s="11" t="s">
+      <c r="E27" s="9" t="s">
         <v>56</v>
       </c>
-      <c r="F27" s="13">
+      <c r="F27" s="10">
         <v>1280219</v>
       </c>
-      <c r="H27" s="11" t="s">
+      <c r="H27" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="I27" s="13">
+      <c r="I27" s="10">
         <v>44470455</v>
       </c>
-      <c r="J27" s="13">
+      <c r="J27" s="10">
         <v>155111022</v>
       </c>
-      <c r="L27" s="14" t="s">
+      <c r="L27" s="11" t="s">
         <v>61</v>
       </c>
-      <c r="M27" s="12">
+      <c r="M27">
         <v>0.12</v>
       </c>
     </row>
     <row r="28" spans="5:13" x14ac:dyDescent="0.3">
-      <c r="E28" s="11" t="s">
+      <c r="E28" s="9" t="s">
         <v>54</v>
       </c>
-      <c r="F28" s="13">
+      <c r="F28" s="10">
         <v>1475057</v>
       </c>
-      <c r="H28" s="11" t="s">
+      <c r="H28" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="I28" s="13">
+      <c r="I28" s="10">
         <v>50827531</v>
       </c>
-      <c r="J28" s="13">
+      <c r="J28" s="10">
         <v>61545441</v>
       </c>
-      <c r="L28" s="11" t="s">
+      <c r="L28" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="M28" s="12">
+      <c r="M28">
         <v>4.99</v>
       </c>
     </row>
     <row r="29" spans="5:13" x14ac:dyDescent="0.3">
-      <c r="E29" s="11" t="s">
+      <c r="E29" s="9" t="s">
         <v>66</v>
       </c>
-      <c r="F29" s="13">
+      <c r="F29" s="10">
         <v>541867</v>
       </c>
-      <c r="H29" s="11" t="s">
+      <c r="H29" s="9" t="s">
         <v>61</v>
       </c>
-      <c r="I29" s="13">
+      <c r="I29" s="10">
         <v>906309</v>
       </c>
-      <c r="J29" s="13">
+      <c r="J29" s="10">
         <v>551414</v>
       </c>
-      <c r="L29" s="14" t="s">
+      <c r="L29" s="11" t="s">
         <v>32</v>
       </c>
-      <c r="M29" s="12">
+      <c r="M29">
         <v>4.99</v>
       </c>
     </row>
     <row r="30" spans="5:13" x14ac:dyDescent="0.3">
-      <c r="E30" s="11" t="s">
+      <c r="E30" s="9" t="s">
         <v>58</v>
       </c>
-      <c r="F30" s="13">
+      <c r="F30" s="10">
         <v>953853</v>
       </c>
-      <c r="H30" s="11" t="s">
+      <c r="H30" s="9" t="s">
         <v>18</v>
       </c>
-      <c r="I30" s="13">
+      <c r="I30" s="10">
         <v>11729609</v>
       </c>
-      <c r="J30" s="13">
+      <c r="J30" s="10">
         <v>92075028</v>
       </c>
-      <c r="L30" s="11" t="s">
+      <c r="L30" s="9" t="s">
         <v>45</v>
       </c>
-      <c r="M30" s="12">
+      <c r="M30">
         <v>2.09</v>
       </c>
     </row>
     <row r="31" spans="5:13" x14ac:dyDescent="0.3">
-      <c r="E31" s="11" t="s">
+      <c r="E31" s="9" t="s">
         <v>33</v>
       </c>
-      <c r="F31" s="13">
+      <c r="F31" s="10">
         <v>20762082</v>
       </c>
-      <c r="H31" s="11" t="s">
+      <c r="H31" s="9" t="s">
         <v>65</v>
       </c>
-      <c r="I31" s="13">
+      <c r="I31" s="10">
         <v>850123</v>
       </c>
-      <c r="J31" s="13">
+      <c r="J31" s="10">
         <v>394341</v>
       </c>
-      <c r="L31" s="14" t="s">
+      <c r="L31" s="11" t="s">
         <v>42</v>
       </c>
-      <c r="M31" s="12">
+      <c r="M31">
         <v>2.09</v>
       </c>
     </row>
     <row r="32" spans="5:13" x14ac:dyDescent="0.3">
-      <c r="E32" s="11" t="s">
+      <c r="E32" s="9" t="s">
         <v>64</v>
       </c>
-      <c r="F32" s="13">
+      <c r="F32" s="10">
         <v>635442</v>
       </c>
-      <c r="H32" s="11" t="s">
+      <c r="H32" s="9" t="s">
         <v>71</v>
       </c>
-      <c r="I32" s="13">
+      <c r="I32" s="10">
         <v>135533</v>
       </c>
-      <c r="J32" s="13">
+      <c r="J32" s="10">
         <v>244411</v>
       </c>
-      <c r="L32" s="11" t="s">
+      <c r="L32" s="9" t="s">
         <v>50</v>
       </c>
-      <c r="M32" s="12">
+      <c r="M32">
         <v>0.56999999999999995</v>
       </c>
     </row>
     <row r="33" spans="5:13" x14ac:dyDescent="0.3">
-      <c r="E33" s="11" t="s">
+      <c r="E33" s="9" t="s">
         <v>41</v>
       </c>
-      <c r="F33" s="13">
+      <c r="F33" s="10">
         <v>13103873</v>
       </c>
-      <c r="H33" s="11" t="s">
+      <c r="H33" s="9" t="s">
         <v>44</v>
       </c>
-      <c r="I33" s="13">
+      <c r="I33" s="10">
         <v>5936538</v>
       </c>
-      <c r="J33" s="13">
+      <c r="J33" s="10">
         <v>19603658</v>
       </c>
-      <c r="L33" s="14" t="s">
+      <c r="L33" s="11" t="s">
         <v>51</v>
       </c>
-      <c r="M33" s="12">
+      <c r="M33">
         <v>0.56999999999999995</v>
       </c>
     </row>
     <row r="34" spans="5:13" x14ac:dyDescent="0.3">
-      <c r="E34" s="11" t="s">
+      <c r="E34" s="9" t="s">
         <v>27</v>
       </c>
-      <c r="F34" s="13">
+      <c r="F34" s="10">
         <v>32997440</v>
       </c>
-      <c r="H34" s="11" t="s">
+      <c r="H34" s="9" t="s">
         <v>38</v>
       </c>
-      <c r="I34" s="13">
+      <c r="I34" s="10">
         <v>7929292</v>
       </c>
-      <c r="J34" s="13">
+      <c r="J34" s="10">
         <v>25036946</v>
       </c>
-      <c r="L34" s="11" t="s">
+      <c r="L34" s="9" t="s">
         <v>47</v>
       </c>
-      <c r="M34" s="12">
+      <c r="M34">
         <v>1.04</v>
       </c>
     </row>
     <row r="35" spans="5:13" x14ac:dyDescent="0.3">
-      <c r="E35" s="11" t="s">
+      <c r="E35" s="9" t="s">
         <v>68</v>
       </c>
-      <c r="F35" s="13">
+      <c r="F35" s="10">
         <v>287507</v>
       </c>
-      <c r="H35" s="11" t="s">
+      <c r="H35" s="9" t="s">
         <v>55</v>
       </c>
-      <c r="I35" s="13">
+      <c r="I35" s="10">
         <v>595036</v>
       </c>
-      <c r="J35" s="13">
+      <c r="J35" s="10">
         <v>2368971</v>
       </c>
-      <c r="L35" s="14" t="s">
+      <c r="L35" s="11" t="s">
         <v>47</v>
       </c>
-      <c r="M35" s="12">
+      <c r="M35">
         <v>1.04</v>
       </c>
     </row>
     <row r="36" spans="5:13" x14ac:dyDescent="0.3">
-      <c r="E36" s="11" t="s">
+      <c r="E36" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="F36" s="13">
+      <c r="F36" s="10">
         <v>36009055</v>
       </c>
-      <c r="H36" s="11" t="s">
+      <c r="H36" s="9" t="s">
         <v>51</v>
       </c>
-      <c r="I36" s="13">
+      <c r="I36" s="10">
         <v>688704</v>
       </c>
-      <c r="J36" s="13">
+      <c r="J36" s="10">
         <v>6167805</v>
       </c>
-      <c r="L36" s="11" t="s">
+      <c r="L36" s="9" t="s">
         <v>37</v>
       </c>
-      <c r="M36" s="12">
+      <c r="M36">
         <v>2.72</v>
       </c>
     </row>
     <row r="37" spans="5:13" x14ac:dyDescent="0.3">
-      <c r="E37" s="11" t="s">
+      <c r="E37" s="9" t="s">
         <v>52</v>
       </c>
-      <c r="F37" s="13">
+      <c r="F37" s="10">
         <v>1799541</v>
       </c>
-      <c r="H37" s="11" t="s">
+      <c r="H37" s="9" t="s">
         <v>73</v>
       </c>
-      <c r="I37" s="13">
+      <c r="I37" s="10">
         <v>159829</v>
       </c>
-      <c r="J37" s="13">
+      <c r="J37" s="10">
         <v>183024</v>
       </c>
-      <c r="L37" s="14" t="s">
+      <c r="L37" s="11" t="s">
         <v>38</v>
       </c>
-      <c r="M37" s="12">
+      <c r="M37">
         <v>2.72</v>
       </c>
     </row>
     <row r="38" spans="5:13" x14ac:dyDescent="0.3">
-      <c r="E38" s="11" t="s">
+      <c r="E38" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="F38" s="13">
+      <c r="F38" s="10">
         <v>95331831</v>
       </c>
-      <c r="H38" s="11" t="s">
+      <c r="H38" s="9" t="s">
         <v>36</v>
       </c>
-      <c r="I38" s="13">
+      <c r="I38" s="10">
         <v>15932171</v>
       </c>
-      <c r="J38" s="13">
+      <c r="J38" s="10">
         <v>17445506</v>
       </c>
-      <c r="L38" s="11" t="s">
+      <c r="L38" s="9" t="s">
         <v>29</v>
       </c>
-      <c r="M38" s="12">
+      <c r="M38">
         <v>5.05</v>
       </c>
     </row>
     <row r="39" spans="5:13" x14ac:dyDescent="0.3">
-      <c r="E39" s="11" t="s">
+      <c r="E39" s="9" t="s">
         <v>48</v>
       </c>
-      <c r="F39" s="13">
+      <c r="F39" s="10">
         <v>4948519</v>
       </c>
-      <c r="H39" s="11" t="s">
+      <c r="H39" s="9" t="s">
         <v>89</v>
       </c>
-      <c r="I39" s="13">
+      <c r="I39" s="10">
         <v>373542974</v>
       </c>
-      <c r="J39" s="13">
+      <c r="J39" s="10">
         <v>833652994</v>
       </c>
-      <c r="L39" s="14" t="s">
+      <c r="L39" s="11" t="s">
         <v>30</v>
       </c>
-      <c r="M39" s="12">
+      <c r="M39">
         <v>5.05</v>
       </c>
     </row>
     <row r="40" spans="5:13" x14ac:dyDescent="0.3">
-      <c r="E40" s="11" t="s">
+      <c r="E40" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="F40" s="13">
+      <c r="F40" s="10">
         <v>44467088</v>
       </c>
-      <c r="L40" s="11" t="s">
+      <c r="L40" s="9" t="s">
         <v>35</v>
       </c>
-      <c r="M40" s="12">
+      <c r="M40">
         <v>2.76</v>
       </c>
     </row>
     <row r="41" spans="5:13" x14ac:dyDescent="0.3">
-      <c r="E41" s="11" t="s">
+      <c r="E41" s="9" t="s">
         <v>89</v>
       </c>
-      <c r="F41" s="13">
+      <c r="F41" s="10">
         <v>587447730</v>
       </c>
-      <c r="L41" s="14" t="s">
+      <c r="L41" s="11" t="s">
         <v>36</v>
       </c>
-      <c r="M41" s="12">
+      <c r="M41">
         <v>2.76</v>
       </c>
     </row>
     <row r="42" spans="5:13" x14ac:dyDescent="0.3">
-      <c r="L42" s="11" t="s">
+      <c r="L42" s="9" t="s">
         <v>76</v>
       </c>
-      <c r="M42" s="12">
+      <c r="M42">
         <v>0.01</v>
       </c>
     </row>
     <row r="43" spans="5:13" x14ac:dyDescent="0.3">
-      <c r="L43" s="14" t="s">
+      <c r="L43" s="11" t="s">
         <v>77</v>
       </c>
-      <c r="M43" s="12">
+      <c r="M43">
         <v>0.01</v>
       </c>
     </row>
     <row r="44" spans="5:13" x14ac:dyDescent="0.3">
-      <c r="L44" s="11" t="s">
+      <c r="L44" s="9" t="s">
         <v>23</v>
       </c>
-      <c r="M44" s="12">
+      <c r="M44">
         <v>6</v>
       </c>
     </row>
     <row r="45" spans="5:13" x14ac:dyDescent="0.3">
-      <c r="L45" s="14" t="s">
+      <c r="L45" s="11" t="s">
         <v>24</v>
       </c>
-      <c r="M45" s="12">
+      <c r="M45">
         <v>6</v>
       </c>
     </row>
     <row r="46" spans="5:13" x14ac:dyDescent="0.3">
-      <c r="L46" s="11" t="s">
+      <c r="L46" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="M46" s="12">
+      <c r="M46">
         <v>9.2799999999999994</v>
       </c>
     </row>
     <row r="47" spans="5:13" x14ac:dyDescent="0.3">
-      <c r="L47" s="14" t="s">
+      <c r="L47" s="11" t="s">
         <v>16</v>
       </c>
-      <c r="M47" s="12">
+      <c r="M47">
         <v>9.2799999999999994</v>
       </c>
     </row>
     <row r="48" spans="5:13" x14ac:dyDescent="0.3">
-      <c r="L48" s="11" t="s">
+      <c r="L48" s="9" t="s">
         <v>56</v>
       </c>
-      <c r="M48" s="12">
+      <c r="M48">
         <v>0.21</v>
       </c>
     </row>
     <row r="49" spans="12:13" x14ac:dyDescent="0.3">
-      <c r="L49" s="14" t="s">
+      <c r="L49" s="11" t="s">
         <v>57</v>
       </c>
-      <c r="M49" s="12">
+      <c r="M49">
         <v>0.21</v>
       </c>
     </row>
     <row r="50" spans="12:13" x14ac:dyDescent="0.3">
-      <c r="L50" s="11" t="s">
+      <c r="L50" s="9" t="s">
         <v>54</v>
       </c>
-      <c r="M50" s="12">
+      <c r="M50">
         <v>0.25</v>
       </c>
     </row>
     <row r="51" spans="12:13" x14ac:dyDescent="0.3">
-      <c r="L51" s="14" t="s">
+      <c r="L51" s="11" t="s">
         <v>55</v>
       </c>
-      <c r="M51" s="12">
+      <c r="M51">
         <v>0.25</v>
       </c>
     </row>
     <row r="52" spans="12:13" x14ac:dyDescent="0.3">
-      <c r="L52" s="11" t="s">
+      <c r="L52" s="9" t="s">
         <v>66</v>
       </c>
-      <c r="M52" s="12">
+      <c r="M52">
         <v>0.09</v>
       </c>
     </row>
     <row r="53" spans="12:13" x14ac:dyDescent="0.3">
-      <c r="L53" s="14" t="s">
+      <c r="L53" s="11" t="s">
         <v>67</v>
       </c>
-      <c r="M53" s="12">
+      <c r="M53">
         <v>0.09</v>
       </c>
     </row>
     <row r="54" spans="12:13" x14ac:dyDescent="0.3">
-      <c r="L54" s="11" t="s">
+      <c r="L54" s="9" t="s">
         <v>58</v>
       </c>
-      <c r="M54" s="12">
+      <c r="M54">
         <v>0.16</v>
       </c>
     </row>
     <row r="55" spans="12:13" x14ac:dyDescent="0.3">
-      <c r="L55" s="14" t="s">
+      <c r="L55" s="11" t="s">
         <v>59</v>
       </c>
-      <c r="M55" s="12">
+      <c r="M55">
         <v>0.16</v>
       </c>
     </row>
     <row r="56" spans="12:13" x14ac:dyDescent="0.3">
-      <c r="L56" s="11" t="s">
+      <c r="L56" s="9" t="s">
         <v>33</v>
       </c>
-      <c r="M56" s="12">
+      <c r="M56">
         <v>3.47</v>
       </c>
     </row>
     <row r="57" spans="12:13" x14ac:dyDescent="0.3">
-      <c r="L57" s="14" t="s">
+      <c r="L57" s="11" t="s">
         <v>34</v>
       </c>
-      <c r="M57" s="12">
+      <c r="M57">
         <v>3.47</v>
       </c>
     </row>
     <row r="58" spans="12:13" x14ac:dyDescent="0.3">
-      <c r="L58" s="11" t="s">
+      <c r="L58" s="9" t="s">
         <v>64</v>
       </c>
-      <c r="M58" s="12">
+      <c r="M58">
         <v>0.1</v>
       </c>
     </row>
     <row r="59" spans="12:13" x14ac:dyDescent="0.3">
-      <c r="L59" s="14" t="s">
+      <c r="L59" s="11" t="s">
         <v>65</v>
       </c>
-      <c r="M59" s="12">
+      <c r="M59">
         <v>0.1</v>
       </c>
     </row>
     <row r="60" spans="12:13" x14ac:dyDescent="0.3">
-      <c r="L60" s="11" t="s">
+      <c r="L60" s="9" t="s">
         <v>41</v>
       </c>
-      <c r="M60" s="12">
+      <c r="M60">
         <v>2.29</v>
       </c>
     </row>
     <row r="61" spans="12:13" x14ac:dyDescent="0.3">
-      <c r="L61" s="14" t="s">
+      <c r="L61" s="11" t="s">
         <v>42</v>
       </c>
-      <c r="M61" s="12">
+      <c r="M61">
         <v>2.29</v>
       </c>
     </row>
     <row r="62" spans="12:13" x14ac:dyDescent="0.3">
-      <c r="L62" s="11" t="s">
+      <c r="L62" s="9" t="s">
         <v>27</v>
       </c>
-      <c r="M62" s="12">
+      <c r="M62">
         <v>5.66</v>
       </c>
     </row>
     <row r="63" spans="12:13" x14ac:dyDescent="0.3">
-      <c r="L63" s="14" t="s">
+      <c r="L63" s="11" t="s">
         <v>28</v>
       </c>
-      <c r="M63" s="12">
+      <c r="M63">
         <v>5.66</v>
       </c>
     </row>
     <row r="64" spans="12:13" x14ac:dyDescent="0.3">
-      <c r="L64" s="11" t="s">
+      <c r="L64" s="9" t="s">
         <v>68</v>
       </c>
-      <c r="M64" s="12">
+      <c r="M64">
         <v>0.05</v>
       </c>
     </row>
     <row r="65" spans="12:13" x14ac:dyDescent="0.3">
-      <c r="L65" s="14" t="s">
+      <c r="L65" s="11" t="s">
         <v>69</v>
       </c>
-      <c r="M65" s="12">
+      <c r="M65">
         <v>0.05</v>
       </c>
     </row>
     <row r="66" spans="12:13" x14ac:dyDescent="0.3">
-      <c r="L66" s="11" t="s">
+      <c r="L66" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="M66" s="12">
+      <c r="M66">
         <v>5.96</v>
       </c>
     </row>
     <row r="67" spans="12:13" x14ac:dyDescent="0.3">
-      <c r="L67" s="14" t="s">
+      <c r="L67" s="11" t="s">
         <v>26</v>
       </c>
-      <c r="M67" s="12">
+      <c r="M67">
         <v>5.96</v>
       </c>
     </row>
     <row r="68" spans="12:13" x14ac:dyDescent="0.3">
-      <c r="L68" s="11" t="s">
+      <c r="L68" s="9" t="s">
         <v>52</v>
       </c>
-      <c r="M68" s="12">
+      <c r="M68">
         <v>0.3</v>
       </c>
     </row>
     <row r="69" spans="12:13" x14ac:dyDescent="0.3">
-      <c r="L69" s="14" t="s">
+      <c r="L69" s="11" t="s">
         <v>53</v>
       </c>
-      <c r="M69" s="12">
+      <c r="M69">
         <v>0.3</v>
       </c>
     </row>
     <row r="70" spans="12:13" x14ac:dyDescent="0.3">
-      <c r="L70" s="11" t="s">
+      <c r="L70" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="M70" s="12">
+      <c r="M70">
         <v>16.5</v>
       </c>
     </row>
     <row r="71" spans="12:13" x14ac:dyDescent="0.3">
-      <c r="L71" s="14" t="s">
+      <c r="L71" s="11" t="s">
         <v>14</v>
       </c>
-      <c r="M71" s="12">
+      <c r="M71">
         <v>16.5</v>
       </c>
     </row>
     <row r="72" spans="12:13" x14ac:dyDescent="0.3">
-      <c r="L72" s="11" t="s">
+      <c r="L72" s="9" t="s">
         <v>48</v>
       </c>
-      <c r="M72" s="12">
+      <c r="M72">
         <v>0.83</v>
       </c>
     </row>
     <row r="73" spans="12:13" x14ac:dyDescent="0.3">
-      <c r="L73" s="14" t="s">
+      <c r="L73" s="11" t="s">
         <v>49</v>
       </c>
-      <c r="M73" s="12">
+      <c r="M73">
         <v>0.83</v>
       </c>
     </row>
     <row r="74" spans="12:13" x14ac:dyDescent="0.3">
-      <c r="L74" s="11" t="s">
+      <c r="L74" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="M74" s="12">
+      <c r="M74">
         <v>7.54</v>
       </c>
     </row>
     <row r="75" spans="12:13" x14ac:dyDescent="0.3">
-      <c r="L75" s="14" t="s">
+      <c r="L75" s="11" t="s">
         <v>20</v>
       </c>
-      <c r="M75" s="12">
+      <c r="M75">
         <v>7.54</v>
       </c>
     </row>
     <row r="76" spans="12:13" x14ac:dyDescent="0.3">
-      <c r="L76" s="11" t="s">
+      <c r="L76" s="9" t="s">
         <v>89</v>
       </c>
-      <c r="M76" s="12">
+      <c r="M76">
         <v>99.99</v>
       </c>
     </row>

</xml_diff>

<commit_message>
update some pivot table in excel
</commit_message>
<xml_diff>
--- a/population.csv.xlsx
+++ b/population.csv.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\My Project\Indian Population Data Analysis\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DA8B4099-5B02-420F-93F1-66877240B4F4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C5ED63F8-AA14-4807-BE25-B77AE7D423CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{FB82829B-6F12-444B-8421-B58D62F0B729}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{FB82829B-6F12-444B-8421-B58D62F0B729}"/>
   </bookViews>
   <sheets>
     <sheet name="population" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
   <calcPr calcId="191029"/>
   <pivotCaches>
     <pivotCache cacheId="0" r:id="rId4"/>
-    <pivotCache cacheId="1" r:id="rId5"/>
+    <pivotCache cacheId="2" r:id="rId5"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
   <metadataTypes count="1">
     <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
   </metadataTypes>
@@ -61,7 +61,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="278" uniqueCount="96">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="281" uniqueCount="97">
   <si>
     <t>Rank</t>
   </si>
@@ -349,6 +349,9 @@
   </si>
   <si>
     <t>Sum of Urban Population</t>
+  </si>
+  <si>
+    <t>Sum of Males</t>
   </si>
 </sst>
 </file>
@@ -888,10 +891,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="36" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="35" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="16" fillId="36" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -1280,7 +1283,43 @@
       </sharedItems>
     </cacheField>
     <cacheField name="Males" numFmtId="3">
-      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="33123" maxValue="104480510"/>
+      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="33123" maxValue="104480510" count="35">
+        <n v="104480510"/>
+        <n v="58243056"/>
+        <n v="54278157"/>
+        <n v="46809027"/>
+        <n v="42442146"/>
+        <n v="37612306"/>
+        <n v="36137975"/>
+        <n v="35550997"/>
+        <n v="30966657"/>
+        <n v="31491260"/>
+        <n v="21212136"/>
+        <n v="16027412"/>
+        <n v="16930315"/>
+        <n v="15939443"/>
+        <n v="14639465"/>
+        <n v="12832895"/>
+        <n v="13494734"/>
+        <n v="8887326"/>
+        <n v="6640662"/>
+        <n v="5137773"/>
+        <n v="3481873"/>
+        <n v="1874376"/>
+        <n v="1491832"/>
+        <n v="1290171"/>
+        <n v="1024649"/>
+        <n v="739140"/>
+        <n v="713912"/>
+        <n v="612511"/>
+        <n v="555339"/>
+        <n v="580663"/>
+        <n v="323070"/>
+        <n v="202871"/>
+        <n v="193760"/>
+        <n v="150301"/>
+        <n v="33123"/>
+      </sharedItems>
     </cacheField>
     <cacheField name="Females" numFmtId="3">
       <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1" minValue="31350" maxValue="95331831"/>
@@ -2164,7 +2203,7 @@
     <x v="0"/>
     <n v="199812341"/>
     <x v="0"/>
-    <n v="104480510"/>
+    <x v="0"/>
     <n v="95331831"/>
     <x v="0"/>
     <x v="0"/>
@@ -2180,7 +2219,7 @@
     <x v="1"/>
     <n v="112374333"/>
     <x v="1"/>
-    <n v="58243056"/>
+    <x v="1"/>
     <n v="54131277"/>
     <x v="1"/>
     <x v="1"/>
@@ -2196,7 +2235,7 @@
     <x v="2"/>
     <n v="104099452"/>
     <x v="2"/>
-    <n v="54278157"/>
+    <x v="2"/>
     <n v="49821295"/>
     <x v="2"/>
     <x v="2"/>
@@ -2212,7 +2251,7 @@
     <x v="3"/>
     <n v="91276115"/>
     <x v="3"/>
-    <n v="46809027"/>
+    <x v="3"/>
     <n v="44467088"/>
     <x v="3"/>
     <x v="3"/>
@@ -2228,7 +2267,7 @@
     <x v="4"/>
     <n v="84580777"/>
     <x v="4"/>
-    <n v="42442146"/>
+    <x v="4"/>
     <n v="42138631"/>
     <x v="4"/>
     <x v="4"/>
@@ -2244,7 +2283,7 @@
     <x v="5"/>
     <n v="72626809"/>
     <x v="5"/>
-    <n v="37612306"/>
+    <x v="5"/>
     <n v="35014503"/>
     <x v="5"/>
     <x v="5"/>
@@ -2260,7 +2299,7 @@
     <x v="6"/>
     <n v="72147030"/>
     <x v="6"/>
-    <n v="36137975"/>
+    <x v="6"/>
     <n v="36009055"/>
     <x v="6"/>
     <x v="6"/>
@@ -2276,7 +2315,7 @@
     <x v="7"/>
     <n v="68548437"/>
     <x v="7"/>
-    <n v="35550997"/>
+    <x v="7"/>
     <n v="32997440"/>
     <x v="7"/>
     <x v="7"/>
@@ -2292,7 +2331,7 @@
     <x v="8"/>
     <n v="61095297"/>
     <x v="8"/>
-    <n v="30966657"/>
+    <x v="8"/>
     <n v="30128640"/>
     <x v="8"/>
     <x v="8"/>
@@ -2308,7 +2347,7 @@
     <x v="9"/>
     <n v="60439692"/>
     <x v="9"/>
-    <n v="31491260"/>
+    <x v="9"/>
     <n v="28948432"/>
     <x v="9"/>
     <x v="9"/>
@@ -2324,7 +2363,7 @@
     <x v="10"/>
     <n v="41974218"/>
     <x v="10"/>
-    <n v="21212136"/>
+    <x v="10"/>
     <n v="20762082"/>
     <x v="10"/>
     <x v="10"/>
@@ -2340,7 +2379,7 @@
     <x v="11"/>
     <n v="33406061"/>
     <x v="11"/>
-    <n v="16027412"/>
+    <x v="11"/>
     <n v="17378649"/>
     <x v="11"/>
     <x v="11"/>
@@ -2356,7 +2395,7 @@
     <x v="12"/>
     <n v="32988134"/>
     <x v="12"/>
-    <n v="16930315"/>
+    <x v="12"/>
     <n v="16057819"/>
     <x v="12"/>
     <x v="12"/>
@@ -2372,7 +2411,7 @@
     <x v="13"/>
     <n v="31205576"/>
     <x v="13"/>
-    <n v="15939443"/>
+    <x v="13"/>
     <n v="15266133"/>
     <x v="13"/>
     <x v="13"/>
@@ -2388,7 +2427,7 @@
     <x v="14"/>
     <n v="27743338"/>
     <x v="14"/>
-    <n v="14639465"/>
+    <x v="14"/>
     <n v="13103873"/>
     <x v="14"/>
     <x v="14"/>
@@ -2404,7 +2443,7 @@
     <x v="15"/>
     <n v="25545198"/>
     <x v="15"/>
-    <n v="12832895"/>
+    <x v="15"/>
     <n v="12712303"/>
     <x v="15"/>
     <x v="15"/>
@@ -2420,7 +2459,7 @@
     <x v="14"/>
     <n v="25351462"/>
     <x v="16"/>
-    <n v="13494734"/>
+    <x v="16"/>
     <n v="11856728"/>
     <x v="16"/>
     <x v="16"/>
@@ -2436,7 +2475,7 @@
     <x v="16"/>
     <n v="16787941"/>
     <x v="17"/>
-    <n v="8887326"/>
+    <x v="17"/>
     <n v="7800615"/>
     <x v="17"/>
     <x v="17"/>
@@ -2452,7 +2491,7 @@
     <x v="17"/>
     <n v="12541302"/>
     <x v="18"/>
-    <n v="6640662"/>
+    <x v="18"/>
     <n v="5900640"/>
     <x v="18"/>
     <x v="18"/>
@@ -2468,7 +2507,7 @@
     <x v="18"/>
     <n v="10086292"/>
     <x v="19"/>
-    <n v="5137773"/>
+    <x v="19"/>
     <n v="4948519"/>
     <x v="19"/>
     <x v="19"/>
@@ -2484,7 +2523,7 @@
     <x v="19"/>
     <n v="6864602"/>
     <x v="20"/>
-    <n v="3481873"/>
+    <x v="20"/>
     <n v="3382729"/>
     <x v="20"/>
     <x v="20"/>
@@ -2500,7 +2539,7 @@
     <x v="20"/>
     <n v="3673917"/>
     <x v="21"/>
-    <n v="1874376"/>
+    <x v="21"/>
     <n v="1799541"/>
     <x v="21"/>
     <x v="21"/>
@@ -2516,7 +2555,7 @@
     <x v="21"/>
     <n v="2966889"/>
     <x v="22"/>
-    <n v="1491832"/>
+    <x v="22"/>
     <n v="1475057"/>
     <x v="22"/>
     <x v="22"/>
@@ -2532,7 +2571,7 @@
     <x v="22"/>
     <n v="2721756"/>
     <x v="23"/>
-    <n v="1290171"/>
+    <x v="23"/>
     <n v="1280219"/>
     <x v="23"/>
     <x v="23"/>
@@ -2548,7 +2587,7 @@
     <x v="23"/>
     <n v="1978502"/>
     <x v="24"/>
-    <n v="1024649"/>
+    <x v="24"/>
     <n v="953853"/>
     <x v="5"/>
     <x v="24"/>
@@ -2564,7 +2603,7 @@
     <x v="24"/>
     <n v="1458545"/>
     <x v="25"/>
-    <n v="739140"/>
+    <x v="25"/>
     <n v="719405"/>
     <x v="8"/>
     <x v="25"/>
@@ -2580,7 +2619,7 @@
     <x v="25"/>
     <n v="1383727"/>
     <x v="26"/>
-    <n v="713912"/>
+    <x v="26"/>
     <n v="669815"/>
     <x v="24"/>
     <x v="26"/>
@@ -2596,7 +2635,7 @@
     <x v="26"/>
     <n v="1247953"/>
     <x v="27"/>
-    <n v="612511"/>
+    <x v="27"/>
     <n v="635442"/>
     <x v="25"/>
     <x v="27"/>
@@ -2612,7 +2651,7 @@
     <x v="27"/>
     <n v="1097206"/>
     <x v="28"/>
-    <n v="555339"/>
+    <x v="28"/>
     <n v="541867"/>
     <x v="26"/>
     <x v="28"/>
@@ -2628,7 +2667,7 @@
     <x v="14"/>
     <n v="1055450"/>
     <x v="28"/>
-    <n v="580663"/>
+    <x v="29"/>
     <n v="474787"/>
     <x v="27"/>
     <x v="29"/>
@@ -2644,7 +2683,7 @@
     <x v="28"/>
     <n v="610577"/>
     <x v="29"/>
-    <n v="323070"/>
+    <x v="30"/>
     <n v="287507"/>
     <x v="28"/>
     <x v="30"/>
@@ -2660,7 +2699,7 @@
     <x v="29"/>
     <n v="380581"/>
     <x v="30"/>
-    <n v="202871"/>
+    <x v="31"/>
     <n v="177710"/>
     <x v="29"/>
     <x v="31"/>
@@ -2676,7 +2715,7 @@
     <x v="30"/>
     <n v="343709"/>
     <x v="30"/>
-    <n v="193760"/>
+    <x v="32"/>
     <n v="149949"/>
     <x v="30"/>
     <x v="32"/>
@@ -2692,7 +2731,7 @@
     <x v="31"/>
     <n v="243247"/>
     <x v="31"/>
-    <n v="150301"/>
+    <x v="33"/>
     <n v="92946"/>
     <x v="31"/>
     <x v="33"/>
@@ -2708,7 +2747,7 @@
     <x v="32"/>
     <n v="64473"/>
     <x v="32"/>
-    <n v="33123"/>
+    <x v="34"/>
     <n v="31350"/>
     <x v="32"/>
     <x v="34"/>
@@ -2722,192 +2761,8 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{80C3E7D3-975D-432E-ACA4-EC6B906FDDBE}" name="PivotTable1" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
-  <location ref="A5:B12" firstHeaderRow="1" firstDataRow="1" firstDataCol="1" rowPageCount="1" colPageCount="1"/>
-  <pivotFields count="14">
-    <pivotField showAll="0"/>
-    <pivotField axis="axisRow" showAll="0">
-      <items count="37">
-        <item x="31"/>
-        <item x="4"/>
-        <item x="26"/>
-        <item x="13"/>
-        <item x="2"/>
-        <item x="29"/>
-        <item x="15"/>
-        <item x="32"/>
-        <item x="33"/>
-        <item x="17"/>
-        <item x="25"/>
-        <item x="9"/>
-        <item x="16"/>
-        <item x="20"/>
-        <item x="18"/>
-        <item x="12"/>
-        <item x="8"/>
-        <item x="11"/>
-        <item x="34"/>
-        <item x="5"/>
-        <item x="1"/>
-        <item x="23"/>
-        <item x="22"/>
-        <item x="28"/>
-        <item x="24"/>
-        <item x="10"/>
-        <item x="27"/>
-        <item x="14"/>
-        <item x="7"/>
-        <item x="30"/>
-        <item x="6"/>
-        <item x="21"/>
-        <item x="0"/>
-        <item x="19"/>
-        <item x="3"/>
-        <item x="35"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0">
-      <items count="35">
-        <item x="31"/>
-        <item x="30"/>
-        <item x="27"/>
-        <item x="17"/>
-        <item x="29"/>
-        <item x="16"/>
-        <item x="18"/>
-        <item x="28"/>
-        <item x="14"/>
-        <item x="0"/>
-        <item x="2"/>
-        <item x="9"/>
-        <item x="7"/>
-        <item x="1"/>
-        <item x="5"/>
-        <item x="24"/>
-        <item x="32"/>
-        <item x="12"/>
-        <item x="3"/>
-        <item x="13"/>
-        <item x="21"/>
-        <item x="19"/>
-        <item x="20"/>
-        <item x="8"/>
-        <item x="26"/>
-        <item x="10"/>
-        <item x="22"/>
-        <item x="15"/>
-        <item x="23"/>
-        <item x="4"/>
-        <item x="6"/>
-        <item x="25"/>
-        <item x="11"/>
-        <item x="33"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField axis="axisPage" multipleItemSelectionAllowed="1" showAll="0">
-      <items count="37">
-        <item h="1" x="2"/>
-        <item h="1" x="26"/>
-        <item h="1" x="7"/>
-        <item h="1" x="12"/>
-        <item h="1" x="4"/>
-        <item h="1" x="18"/>
-        <item h="1" x="0"/>
-        <item h="1" x="5"/>
-        <item h="1" x="15"/>
-        <item h="1" x="13"/>
-        <item h="1" x="10"/>
-        <item h="1" x="22"/>
-        <item h="1" x="8"/>
-        <item h="1" x="16"/>
-        <item x="14"/>
-        <item x="32"/>
-        <item h="1" x="3"/>
-        <item h="1" x="9"/>
-        <item h="1" x="23"/>
-        <item h="1" x="24"/>
-        <item x="19"/>
-        <item h="1" x="6"/>
-        <item h="1" x="30"/>
-        <item h="1" x="1"/>
-        <item h="1" x="20"/>
-        <item h="1" x="27"/>
-        <item h="1" x="29"/>
-        <item h="1" x="17"/>
-        <item x="31"/>
-        <item h="1" x="33"/>
-        <item h="1" x="21"/>
-        <item h="1" x="25"/>
-        <item h="1" x="28"/>
-        <item x="34"/>
-        <item x="11"/>
-        <item h="1" x="35"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField dataField="1" showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-  </pivotFields>
-  <rowFields count="1">
-    <field x="1"/>
-  </rowFields>
-  <rowItems count="7">
-    <i>
-      <x/>
-    </i>
-    <i>
-      <x v="7"/>
-    </i>
-    <i>
-      <x v="17"/>
-    </i>
-    <i>
-      <x v="18"/>
-    </i>
-    <i>
-      <x v="27"/>
-    </i>
-    <i>
-      <x v="33"/>
-    </i>
-    <i t="grand">
-      <x/>
-    </i>
-  </rowItems>
-  <colItems count="1">
-    <i/>
-  </colItems>
-  <pageFields count="1">
-    <pageField fld="8" hier="-1"/>
-  </pageFields>
-  <dataFields count="1">
-    <dataField name="Sum of Rural Population" fld="9" baseField="0" baseItem="0"/>
-  </dataFields>
-  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
-      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
-    </ext>
-    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
-      <xpdl:pivotTableDefinition16/>
-    </ext>
-  </extLst>
-</pivotTableDefinition>
-</file>
-
-<file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{9F7B912B-B7BC-4364-BBA6-38B4B0148DFC}" name="PivotTable4" cacheId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
-  <location ref="L5:M76" firstHeaderRow="1" firstDataRow="1" firstDataCol="1" rowPageCount="1" colPageCount="1"/>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{9F7B912B-B7BC-4364-BBA6-38B4B0148DFC}" name="PivotTable4" cacheId="2" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+  <location ref="M5:N76" firstHeaderRow="1" firstDataRow="1" firstDataCol="1" rowPageCount="1" colPageCount="1"/>
   <pivotFields count="14">
     <pivotField showAll="0"/>
     <pivotField axis="axisRow" showAll="0">
@@ -3316,9 +3171,9 @@
 </pivotTableDefinition>
 </file>
 
-<file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{51E9E64C-34E6-49FF-ABC4-DCBA46C9B4F0}" name="PivotTable3" cacheId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
-  <location ref="H5:J39" firstHeaderRow="0" firstDataRow="1" firstDataCol="1" rowPageCount="1" colPageCount="1"/>
+<file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{51E9E64C-34E6-49FF-ABC4-DCBA46C9B4F0}" name="PivotTable3" cacheId="2" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+  <location ref="I5:K39" firstHeaderRow="0" firstDataRow="1" firstDataCol="1" rowPageCount="1" colPageCount="1"/>
   <pivotFields count="14">
     <pivotField showAll="0"/>
     <pivotField showAll="0">
@@ -3585,9 +3440,9 @@
 </pivotTableDefinition>
 </file>
 
-<file path=xl/pivotTables/pivotTable4.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{283C2D54-EA66-46DD-A52C-DBEC61E2F94E}" name="PivotTable2" cacheId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
-  <location ref="E5:F41" firstHeaderRow="1" firstDataRow="1" firstDataCol="1" rowPageCount="1" colPageCount="1"/>
+<file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{283C2D54-EA66-46DD-A52C-DBEC61E2F94E}" name="PivotTable2" cacheId="2" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+  <location ref="E5:G41" firstHeaderRow="0" firstDataRow="1" firstDataCol="1" rowPageCount="2" colPageCount="1"/>
   <pivotFields count="14">
     <pivotField showAll="0">
       <items count="36">
@@ -3709,9 +3564,48 @@
     </pivotField>
     <pivotField numFmtId="3" showAll="0"/>
     <pivotField showAll="0"/>
-    <pivotField numFmtId="3" showAll="0"/>
+    <pivotField dataField="1" numFmtId="3" showAll="0">
+      <items count="36">
+        <item x="34"/>
+        <item x="33"/>
+        <item x="32"/>
+        <item x="31"/>
+        <item x="30"/>
+        <item x="28"/>
+        <item x="29"/>
+        <item x="27"/>
+        <item x="26"/>
+        <item x="25"/>
+        <item x="24"/>
+        <item x="23"/>
+        <item x="22"/>
+        <item x="21"/>
+        <item x="20"/>
+        <item x="19"/>
+        <item x="18"/>
+        <item x="17"/>
+        <item x="15"/>
+        <item x="16"/>
+        <item x="14"/>
+        <item x="13"/>
+        <item x="11"/>
+        <item x="12"/>
+        <item x="10"/>
+        <item x="8"/>
+        <item x="9"/>
+        <item x="7"/>
+        <item x="6"/>
+        <item x="5"/>
+        <item x="4"/>
+        <item x="3"/>
+        <item x="2"/>
+        <item x="1"/>
+        <item x="0"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
     <pivotField dataField="1" numFmtId="3" showAll="0"/>
-    <pivotField axis="axisPage" multipleItemSelectionAllowed="1" showAll="0">
+    <pivotField multipleItemSelectionAllowed="1" showAll="0">
       <items count="34">
         <item x="31"/>
         <item x="30"/>
@@ -3789,8 +3683,86 @@
         <item t="default"/>
       </items>
     </pivotField>
-    <pivotField numFmtId="3" showAll="0"/>
-    <pivotField numFmtId="3" showAll="0"/>
+    <pivotField axis="axisPage" numFmtId="3" showAll="0">
+      <items count="36">
+        <item x="34"/>
+        <item x="29"/>
+        <item x="33"/>
+        <item x="32"/>
+        <item x="31"/>
+        <item x="27"/>
+        <item x="30"/>
+        <item x="28"/>
+        <item x="25"/>
+        <item x="17"/>
+        <item x="26"/>
+        <item x="24"/>
+        <item x="23"/>
+        <item x="22"/>
+        <item x="21"/>
+        <item x="20"/>
+        <item x="19"/>
+        <item x="18"/>
+        <item x="16"/>
+        <item x="14"/>
+        <item x="11"/>
+        <item x="15"/>
+        <item x="12"/>
+        <item x="13"/>
+        <item x="9"/>
+        <item x="10"/>
+        <item x="6"/>
+        <item x="8"/>
+        <item x="7"/>
+        <item x="5"/>
+        <item x="4"/>
+        <item x="1"/>
+        <item x="3"/>
+        <item x="2"/>
+        <item x="0"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField axis="axisPage" numFmtId="3" showAll="0">
+      <items count="36">
+        <item x="34"/>
+        <item x="31"/>
+        <item x="30"/>
+        <item x="32"/>
+        <item x="33"/>
+        <item x="26"/>
+        <item x="28"/>
+        <item x="24"/>
+        <item x="22"/>
+        <item x="20"/>
+        <item x="23"/>
+        <item x="27"/>
+        <item x="25"/>
+        <item x="21"/>
+        <item x="29"/>
+        <item x="19"/>
+        <item x="18"/>
+        <item x="13"/>
+        <item x="15"/>
+        <item x="10"/>
+        <item x="12"/>
+        <item x="16"/>
+        <item x="14"/>
+        <item x="2"/>
+        <item x="17"/>
+        <item x="11"/>
+        <item x="7"/>
+        <item x="5"/>
+        <item x="8"/>
+        <item x="9"/>
+        <item x="4"/>
+        <item x="3"/>
+        <item x="6"/>
+        <item x="0"/>
+        <item x="1"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
     <pivotField showAll="0"/>
     <pivotField showAll="0"/>
     <pivotField showAll="0"/>
@@ -3908,14 +3880,208 @@
       <x/>
     </i>
   </rowItems>
+  <colFields count="1">
+    <field x="-2"/>
+  </colFields>
+  <colItems count="2">
+    <i>
+      <x/>
+    </i>
+    <i i="1">
+      <x v="1"/>
+    </i>
+  </colItems>
+  <pageFields count="2">
+    <pageField fld="9" hier="-1"/>
+    <pageField fld="10" hier="-1"/>
+  </pageFields>
+  <dataFields count="2">
+    <dataField name="Sum of Females" fld="6" baseField="0" baseItem="0" numFmtId="3"/>
+    <dataField name="Sum of Males" fld="5" baseField="0" baseItem="0" numFmtId="3"/>
+  </dataFields>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
+<file path=xl/pivotTables/pivotTable4.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{80C3E7D3-975D-432E-ACA4-EC6B906FDDBE}" name="PivotTable1" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+  <location ref="A5:B12" firstHeaderRow="1" firstDataRow="1" firstDataCol="1" rowPageCount="1" colPageCount="1"/>
+  <pivotFields count="14">
+    <pivotField showAll="0"/>
+    <pivotField axis="axisRow" showAll="0">
+      <items count="37">
+        <item x="31"/>
+        <item x="4"/>
+        <item x="26"/>
+        <item x="13"/>
+        <item x="2"/>
+        <item x="29"/>
+        <item x="15"/>
+        <item x="32"/>
+        <item x="33"/>
+        <item x="17"/>
+        <item x="25"/>
+        <item x="9"/>
+        <item x="16"/>
+        <item x="20"/>
+        <item x="18"/>
+        <item x="12"/>
+        <item x="8"/>
+        <item x="11"/>
+        <item x="34"/>
+        <item x="5"/>
+        <item x="1"/>
+        <item x="23"/>
+        <item x="22"/>
+        <item x="28"/>
+        <item x="24"/>
+        <item x="10"/>
+        <item x="27"/>
+        <item x="14"/>
+        <item x="7"/>
+        <item x="30"/>
+        <item x="6"/>
+        <item x="21"/>
+        <item x="0"/>
+        <item x="19"/>
+        <item x="3"/>
+        <item x="35"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0">
+      <items count="35">
+        <item x="31"/>
+        <item x="30"/>
+        <item x="27"/>
+        <item x="17"/>
+        <item x="29"/>
+        <item x="16"/>
+        <item x="18"/>
+        <item x="28"/>
+        <item x="14"/>
+        <item x="0"/>
+        <item x="2"/>
+        <item x="9"/>
+        <item x="7"/>
+        <item x="1"/>
+        <item x="5"/>
+        <item x="24"/>
+        <item x="32"/>
+        <item x="12"/>
+        <item x="3"/>
+        <item x="13"/>
+        <item x="21"/>
+        <item x="19"/>
+        <item x="20"/>
+        <item x="8"/>
+        <item x="26"/>
+        <item x="10"/>
+        <item x="22"/>
+        <item x="15"/>
+        <item x="23"/>
+        <item x="4"/>
+        <item x="6"/>
+        <item x="25"/>
+        <item x="11"/>
+        <item x="33"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField axis="axisPage" multipleItemSelectionAllowed="1" showAll="0">
+      <items count="37">
+        <item h="1" x="2"/>
+        <item h="1" x="26"/>
+        <item h="1" x="7"/>
+        <item h="1" x="12"/>
+        <item h="1" x="4"/>
+        <item h="1" x="18"/>
+        <item h="1" x="0"/>
+        <item h="1" x="5"/>
+        <item h="1" x="15"/>
+        <item h="1" x="13"/>
+        <item h="1" x="10"/>
+        <item h="1" x="22"/>
+        <item h="1" x="8"/>
+        <item h="1" x="16"/>
+        <item x="14"/>
+        <item x="32"/>
+        <item h="1" x="3"/>
+        <item h="1" x="9"/>
+        <item h="1" x="23"/>
+        <item h="1" x="24"/>
+        <item x="19"/>
+        <item h="1" x="6"/>
+        <item h="1" x="30"/>
+        <item h="1" x="1"/>
+        <item h="1" x="20"/>
+        <item h="1" x="27"/>
+        <item h="1" x="29"/>
+        <item h="1" x="17"/>
+        <item x="31"/>
+        <item h="1" x="33"/>
+        <item h="1" x="21"/>
+        <item h="1" x="25"/>
+        <item h="1" x="28"/>
+        <item x="34"/>
+        <item x="11"/>
+        <item h="1" x="35"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField dataField="1" showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+  </pivotFields>
+  <rowFields count="1">
+    <field x="1"/>
+  </rowFields>
+  <rowItems count="7">
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="7"/>
+    </i>
+    <i>
+      <x v="17"/>
+    </i>
+    <i>
+      <x v="18"/>
+    </i>
+    <i>
+      <x v="27"/>
+    </i>
+    <i>
+      <x v="33"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
   <colItems count="1">
     <i/>
   </colItems>
   <pageFields count="1">
-    <pageField fld="7" hier="-1"/>
+    <pageField fld="8" hier="-1"/>
   </pageFields>
   <dataFields count="1">
-    <dataField name="Sum of Females" fld="6" baseField="0" baseItem="0" numFmtId="3"/>
+    <dataField name="Sum of Rural Population" fld="9" baseField="0" baseItem="0"/>
   </dataFields>
   <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
   <extLst>
@@ -5875,19 +6041,19 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="A2" s="12" t="s">
+      <c r="A2" s="13" t="s">
         <v>79</v>
       </c>
-      <c r="B2" s="12"/>
-      <c r="C2" s="12"/>
-      <c r="E2" s="12" t="s">
+      <c r="B2" s="13"/>
+      <c r="C2" s="13"/>
+      <c r="E2" s="13" t="s">
         <v>82</v>
       </c>
-      <c r="F2" s="12"/>
-      <c r="H2" s="12" t="s">
+      <c r="F2" s="13"/>
+      <c r="H2" s="13" t="s">
         <v>85</v>
       </c>
-      <c r="I2" s="12"/>
+      <c r="I2" s="13"/>
       <c r="L2" s="7" t="s">
         <v>1</v>
       </c>
@@ -5929,22 +6095,22 @@
       </c>
     </row>
     <row r="3" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="A3" s="13">
+      <c r="A3" s="12">
         <f>MAX(population!E2:E36)</f>
         <v>16.5</v>
       </c>
-      <c r="B3" s="13"/>
-      <c r="C3" s="13"/>
-      <c r="E3" s="13">
+      <c r="B3" s="12"/>
+      <c r="C3" s="12"/>
+      <c r="E3" s="12">
         <f>MAX(population!H2:H36)</f>
         <v>1084</v>
       </c>
-      <c r="F3" s="13"/>
-      <c r="H3" s="13">
+      <c r="F3" s="12"/>
+      <c r="H3" s="12">
         <f>MAX(population!I2:I36)</f>
         <v>94</v>
       </c>
-      <c r="I3" s="13"/>
+      <c r="I3" s="12"/>
       <c r="L3" s="6" t="s">
         <v>13</v>
       </c>
@@ -6029,19 +6195,19 @@
       </c>
     </row>
     <row r="5" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="A5" s="12" t="s">
+      <c r="A5" s="13" t="s">
         <v>80</v>
       </c>
-      <c r="B5" s="12"/>
-      <c r="C5" s="12"/>
-      <c r="E5" s="12" t="s">
+      <c r="B5" s="13"/>
+      <c r="C5" s="13"/>
+      <c r="E5" s="13" t="s">
         <v>83</v>
       </c>
-      <c r="F5" s="12"/>
-      <c r="H5" s="12" t="s">
+      <c r="F5" s="13"/>
+      <c r="H5" s="13" t="s">
         <v>86</v>
       </c>
-      <c r="I5" s="12"/>
+      <c r="I5" s="13"/>
       <c r="L5" s="6" t="s">
         <v>54</v>
       </c>
@@ -6084,22 +6250,22 @@
       </c>
     </row>
     <row r="6" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="A6" s="13">
+      <c r="A6" s="12">
         <f>MIN(population!E2:E36)</f>
         <v>0.01</v>
       </c>
-      <c r="B6" s="13"/>
-      <c r="C6" s="13"/>
-      <c r="E6" s="13">
+      <c r="B6" s="12"/>
+      <c r="C6" s="12"/>
+      <c r="E6" s="12">
         <f>MIN(population!H2:H36)</f>
         <v>618</v>
       </c>
-      <c r="F6" s="13"/>
-      <c r="H6" s="13">
+      <c r="F6" s="12"/>
+      <c r="H6" s="12">
         <f>MIN(population!I2:I36)</f>
         <v>61.8</v>
       </c>
-      <c r="I6" s="13"/>
+      <c r="I6" s="12"/>
       <c r="L6" s="6" t="s">
         <v>68</v>
       </c>
@@ -6184,19 +6350,19 @@
       </c>
     </row>
     <row r="8" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="A8" s="12" t="s">
+      <c r="A8" s="13" t="s">
         <v>81</v>
       </c>
-      <c r="B8" s="12"/>
-      <c r="C8" s="12"/>
-      <c r="E8" s="12" t="s">
+      <c r="B8" s="13"/>
+      <c r="C8" s="13"/>
+      <c r="E8" s="13" t="s">
         <v>84</v>
       </c>
-      <c r="F8" s="12"/>
-      <c r="H8" s="12" t="s">
+      <c r="F8" s="13"/>
+      <c r="H8" s="13" t="s">
         <v>87</v>
       </c>
-      <c r="I8" s="12"/>
+      <c r="I8" s="13"/>
       <c r="L8" s="6" t="s">
         <v>62</v>
       </c>
@@ -6239,22 +6405,22 @@
       </c>
     </row>
     <row r="9" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="A9" s="13">
+      <c r="A9" s="12">
         <f>AVERAGE(population!E2:E36)</f>
         <v>2.8568571428571428</v>
       </c>
-      <c r="B9" s="13"/>
-      <c r="C9" s="13"/>
-      <c r="E9" s="13">
+      <c r="B9" s="12"/>
+      <c r="C9" s="12"/>
+      <c r="E9" s="12">
         <f>AVERAGE(population!H2:H36)</f>
         <v>931.2285714285714</v>
       </c>
-      <c r="F9" s="13"/>
-      <c r="H9" s="13">
+      <c r="F9" s="12"/>
+      <c r="H9" s="12">
         <f>AVERAGE(population!I11)</f>
         <v>78.03</v>
       </c>
-      <c r="I9" s="13"/>
+      <c r="I9" s="12"/>
       <c r="L9" s="6" t="s">
         <v>66</v>
       </c>
@@ -6298,12 +6464,6 @@
     </row>
   </sheetData>
   <mergeCells count="18">
-    <mergeCell ref="A9:C9"/>
-    <mergeCell ref="A2:C2"/>
-    <mergeCell ref="A3:C3"/>
-    <mergeCell ref="A5:C5"/>
-    <mergeCell ref="A6:C6"/>
-    <mergeCell ref="A8:C8"/>
     <mergeCell ref="H9:I9"/>
     <mergeCell ref="E2:F2"/>
     <mergeCell ref="E3:F3"/>
@@ -6316,6 +6476,12 @@
     <mergeCell ref="H5:I5"/>
     <mergeCell ref="H6:I6"/>
     <mergeCell ref="H8:I8"/>
+    <mergeCell ref="A9:C9"/>
+    <mergeCell ref="A2:C2"/>
+    <mergeCell ref="A3:C3"/>
+    <mergeCell ref="A5:C5"/>
+    <mergeCell ref="A6:C6"/>
+    <mergeCell ref="A8:C8"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
@@ -6324,7 +6490,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{881F210B-A9CA-4D54-9D0F-4913621E3B09}">
-  <dimension ref="A3:M76"/>
+  <dimension ref="A2:N76"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="25.109375" bestFit="1" customWidth="1"/>
@@ -6332,47 +6498,56 @@
     <col min="5" max="5" width="25.109375" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="14.21875" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="26.109375" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="17.77734375" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="21.6640625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="20.88671875" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="18.33203125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="27.77734375" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="24.5546875" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="6.44140625" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="9.21875" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="7" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="13.21875" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="10.44140625" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="7.77734375" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="6.88671875" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="9" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="5.33203125" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="6.44140625" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="11.5546875" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="7.88671875" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="10.21875" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="6.88671875" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="7.77734375" bestFit="1" customWidth="1"/>
-    <col min="29" max="29" width="7" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="17.88671875" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="8.5546875" bestFit="1" customWidth="1"/>
-    <col min="32" max="33" width="7.33203125" bestFit="1" customWidth="1"/>
-    <col min="34" max="34" width="8.21875" bestFit="1" customWidth="1"/>
-    <col min="35" max="35" width="7.77734375" bestFit="1" customWidth="1"/>
-    <col min="36" max="36" width="6.21875" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="6" bestFit="1" customWidth="1"/>
-    <col min="38" max="38" width="11" bestFit="1" customWidth="1"/>
-    <col min="39" max="39" width="8.6640625" bestFit="1" customWidth="1"/>
-    <col min="40" max="40" width="7" bestFit="1" customWidth="1"/>
-    <col min="41" max="41" width="6.6640625" bestFit="1" customWidth="1"/>
-    <col min="42" max="42" width="7.6640625" bestFit="1" customWidth="1"/>
-    <col min="43" max="43" width="6.88671875" bestFit="1" customWidth="1"/>
-    <col min="44" max="44" width="7.88671875" bestFit="1" customWidth="1"/>
-    <col min="45" max="45" width="18.33203125" bestFit="1" customWidth="1"/>
-    <col min="46" max="46" width="10.5546875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="26.109375" customWidth="1"/>
+    <col min="9" max="9" width="17.77734375" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="21.6640625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="20.88671875" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="18.33203125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="27.77734375" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="24.5546875" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="6.44140625" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="9.21875" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="7" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="13.21875" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="10.44140625" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="7.77734375" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="6.88671875" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="9" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="5.33203125" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="6.44140625" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="11.5546875" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="7.88671875" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="10.21875" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="6.88671875" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="7.77734375" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="7" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="17.88671875" bestFit="1" customWidth="1"/>
+    <col min="32" max="32" width="8.5546875" bestFit="1" customWidth="1"/>
+    <col min="33" max="34" width="7.33203125" bestFit="1" customWidth="1"/>
+    <col min="35" max="35" width="8.21875" bestFit="1" customWidth="1"/>
+    <col min="36" max="36" width="7.77734375" bestFit="1" customWidth="1"/>
+    <col min="37" max="37" width="6.21875" bestFit="1" customWidth="1"/>
+    <col min="38" max="38" width="6" bestFit="1" customWidth="1"/>
+    <col min="39" max="39" width="11" bestFit="1" customWidth="1"/>
+    <col min="40" max="40" width="8.6640625" bestFit="1" customWidth="1"/>
+    <col min="41" max="41" width="7" bestFit="1" customWidth="1"/>
+    <col min="42" max="42" width="6.6640625" bestFit="1" customWidth="1"/>
+    <col min="43" max="43" width="7.6640625" bestFit="1" customWidth="1"/>
+    <col min="44" max="44" width="6.88671875" bestFit="1" customWidth="1"/>
+    <col min="45" max="45" width="7.88671875" bestFit="1" customWidth="1"/>
+    <col min="46" max="46" width="18.33203125" bestFit="1" customWidth="1"/>
+    <col min="47" max="47" width="10.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:14" x14ac:dyDescent="0.3">
+      <c r="E2" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="F2" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="3" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A3" s="8" t="s">
         <v>7</v>
       </c>
@@ -6380,25 +6555,25 @@
         <v>92</v>
       </c>
       <c r="E3" s="8" t="s">
-        <v>78</v>
+        <v>9</v>
       </c>
       <c r="F3" t="s">
         <v>91</v>
       </c>
-      <c r="H3" s="8" t="s">
+      <c r="I3" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="I3" t="s">
+      <c r="J3" t="s">
         <v>91</v>
       </c>
-      <c r="L3" s="8" t="s">
+      <c r="M3" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="M3" t="s">
+      <c r="N3" t="s">
         <v>91</v>
       </c>
     </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A5" s="8" t="s">
         <v>88</v>
       </c>
@@ -6411,23 +6586,26 @@
       <c r="F5" t="s">
         <v>93</v>
       </c>
-      <c r="H5" s="8" t="s">
+      <c r="G5" t="s">
+        <v>96</v>
+      </c>
+      <c r="I5" s="8" t="s">
         <v>88</v>
       </c>
-      <c r="I5" t="s">
+      <c r="J5" t="s">
         <v>95</v>
       </c>
-      <c r="J5" t="s">
+      <c r="K5" t="s">
         <v>90</v>
       </c>
-      <c r="L5" s="8" t="s">
+      <c r="M5" s="8" t="s">
         <v>88</v>
       </c>
-      <c r="M5" t="s">
+      <c r="N5" t="s">
         <v>94</v>
       </c>
     </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A6" s="9" t="s">
         <v>70</v>
       </c>
@@ -6440,23 +6618,27 @@
       <c r="F6" s="10">
         <v>177710</v>
       </c>
-      <c r="H6" s="9" t="s">
+      <c r="G6" s="10">
+        <v>202871</v>
+      </c>
+      <c r="H6" s="10"/>
+      <c r="I6" s="9" t="s">
         <v>53</v>
       </c>
-      <c r="I6" s="10">
+      <c r="J6" s="10">
         <v>960981</v>
       </c>
-      <c r="J6" s="10">
+      <c r="K6" s="10">
         <v>2710051</v>
       </c>
-      <c r="L6" s="9" t="s">
+      <c r="M6" s="9" t="s">
         <v>70</v>
       </c>
-      <c r="M6">
+      <c r="N6">
         <v>0.03</v>
       </c>
     </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A7" s="9" t="s">
         <v>72</v>
       </c>
@@ -6469,23 +6651,27 @@
       <c r="F7" s="10">
         <v>42138631</v>
       </c>
-      <c r="H7" s="9" t="s">
+      <c r="G7" s="10">
+        <v>42442146</v>
+      </c>
+      <c r="H7" s="10"/>
+      <c r="I7" s="9" t="s">
         <v>67</v>
       </c>
-      <c r="I7" s="10">
+      <c r="J7" s="10">
         <v>561997</v>
       </c>
-      <c r="J7" s="10">
+      <c r="K7" s="10">
         <v>529037</v>
       </c>
-      <c r="L7" s="11" t="s">
+      <c r="M7" s="11" t="s">
         <v>71</v>
       </c>
-      <c r="M7">
+      <c r="N7">
         <v>0.03</v>
       </c>
     </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A8" s="9" t="s">
         <v>35</v>
       </c>
@@ -6498,23 +6684,27 @@
       <c r="F8" s="10">
         <v>669815</v>
       </c>
-      <c r="H8" s="9" t="s">
+      <c r="G8" s="10">
+        <v>713912</v>
+      </c>
+      <c r="H8" s="10"/>
+      <c r="I8" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="I8" s="10">
+      <c r="J8" s="10">
         <v>23578175</v>
       </c>
-      <c r="J8" s="10">
+      <c r="K8" s="10">
         <v>37552529</v>
       </c>
-      <c r="L8" s="9" t="s">
+      <c r="M8" s="9" t="s">
         <v>21</v>
       </c>
-      <c r="M8">
+      <c r="N8">
         <v>6.99</v>
       </c>
     </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A9" s="9" t="s">
         <v>76</v>
       </c>
@@ -6527,23 +6717,27 @@
       <c r="F9" s="10">
         <v>15266133</v>
       </c>
-      <c r="H9" s="9" t="s">
+      <c r="G9" s="10">
+        <v>15939443</v>
+      </c>
+      <c r="H9" s="10"/>
+      <c r="I9" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="I9" s="10">
+      <c r="J9" s="10">
         <v>20059666</v>
       </c>
-      <c r="J9" s="10">
+      <c r="K9" s="10">
         <v>52537899</v>
       </c>
-      <c r="L9" s="11" t="s">
+      <c r="M9" s="11" t="s">
         <v>22</v>
       </c>
-      <c r="M9">
+      <c r="N9">
         <v>6.99</v>
       </c>
     </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A10" s="9" t="s">
         <v>41</v>
       </c>
@@ -6556,23 +6750,27 @@
       <c r="F10" s="10">
         <v>49821295</v>
       </c>
-      <c r="H10" s="9" t="s">
+      <c r="G10" s="10">
+        <v>54278157</v>
+      </c>
+      <c r="H10" s="10"/>
+      <c r="I10" s="9" t="s">
         <v>34</v>
       </c>
-      <c r="I10" s="10">
+      <c r="J10" s="10">
         <v>6996124</v>
       </c>
-      <c r="J10" s="10">
+      <c r="K10" s="10">
         <v>34951234</v>
       </c>
-      <c r="L10" s="9" t="s">
+      <c r="M10" s="9" t="s">
         <v>62</v>
       </c>
-      <c r="M10">
+      <c r="N10">
         <v>0.11</v>
       </c>
     </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A11" s="9" t="s">
         <v>48</v>
       </c>
@@ -6585,23 +6783,27 @@
       <c r="F11" s="10">
         <v>474787</v>
       </c>
-      <c r="H11" s="9" t="s">
+      <c r="G11" s="10">
+        <v>580663</v>
+      </c>
+      <c r="H11" s="10"/>
+      <c r="I11" s="9" t="s">
         <v>42</v>
       </c>
-      <c r="I11" s="10">
+      <c r="J11" s="10">
         <v>20234706</v>
       </c>
-      <c r="J11" s="10">
+      <c r="K11" s="10">
         <v>33877297</v>
       </c>
-      <c r="L11" s="11" t="s">
+      <c r="M11" s="11" t="s">
         <v>63</v>
       </c>
-      <c r="M11">
+      <c r="N11">
         <v>0.11</v>
       </c>
     </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A12" s="9" t="s">
         <v>89</v>
       </c>
@@ -6614,948 +6816,1068 @@
       <c r="F12" s="10">
         <v>12712303</v>
       </c>
-      <c r="H12" s="9" t="s">
+      <c r="G12" s="10">
+        <v>12832895</v>
+      </c>
+      <c r="H12" s="10"/>
+      <c r="I12" s="9" t="s">
         <v>26</v>
       </c>
-      <c r="I12" s="10">
+      <c r="J12" s="10">
         <v>34949729</v>
       </c>
-      <c r="J12" s="10">
+      <c r="K12" s="10">
         <v>37189229</v>
       </c>
-      <c r="L12" s="9" t="s">
+      <c r="M12" s="9" t="s">
         <v>39</v>
       </c>
-      <c r="M12">
+      <c r="N12">
         <v>2.58</v>
       </c>
     </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:14" x14ac:dyDescent="0.3">
       <c r="E13" s="9" t="s">
         <v>72</v>
       </c>
       <c r="F13" s="10">
         <v>149949</v>
       </c>
-      <c r="H13" s="9" t="s">
+      <c r="G13" s="10">
+        <v>193760</v>
+      </c>
+      <c r="H13" s="10"/>
+      <c r="I13" s="9" t="s">
         <v>75</v>
       </c>
-      <c r="I13" s="10">
+      <c r="J13" s="10">
         <v>182580</v>
       </c>
-      <c r="J13" s="10">
+      <c r="K13" s="10">
         <v>60331</v>
       </c>
-      <c r="L13" s="11" t="s">
+      <c r="M13" s="11" t="s">
         <v>40</v>
       </c>
-      <c r="M13">
+      <c r="N13">
         <v>2.58</v>
       </c>
     </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:14" x14ac:dyDescent="0.3">
       <c r="E14" s="9" t="s">
         <v>74</v>
       </c>
       <c r="F14" s="10">
         <v>92946</v>
       </c>
-      <c r="H14" s="9" t="s">
+      <c r="G14" s="10">
+        <v>150301</v>
+      </c>
+      <c r="H14" s="10"/>
+      <c r="I14" s="9" t="s">
         <v>49</v>
       </c>
-      <c r="I14" s="10">
+      <c r="J14" s="10">
         <v>3091169</v>
       </c>
-      <c r="J14" s="10">
+      <c r="K14" s="10">
         <v>7025583</v>
       </c>
-      <c r="L14" s="9" t="s">
+      <c r="M14" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="M14">
+      <c r="N14">
         <v>8.6</v>
       </c>
     </row>
-    <row r="15" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:14" x14ac:dyDescent="0.3">
       <c r="E15" s="9" t="s">
         <v>46</v>
       </c>
       <c r="F15" s="10">
         <v>7800615</v>
       </c>
-      <c r="H15" s="9" t="s">
+      <c r="G15" s="10">
+        <v>8887326</v>
+      </c>
+      <c r="H15" s="10"/>
+      <c r="I15" s="9" t="s">
         <v>46</v>
       </c>
-      <c r="I15" s="10">
+      <c r="J15" s="10">
         <v>12905780</v>
       </c>
-      <c r="J15" s="10">
+      <c r="K15" s="10">
         <v>944727</v>
       </c>
-      <c r="L15" s="11" t="s">
+      <c r="M15" s="11" t="s">
         <v>18</v>
       </c>
-      <c r="M15">
+      <c r="N15">
         <v>8.6</v>
       </c>
     </row>
-    <row r="16" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:14" x14ac:dyDescent="0.3">
       <c r="E16" s="9" t="s">
         <v>60</v>
       </c>
       <c r="F16" s="10">
         <v>719405</v>
       </c>
-      <c r="H16" s="9" t="s">
+      <c r="G16" s="10">
+        <v>739140</v>
+      </c>
+      <c r="H16" s="10"/>
+      <c r="I16" s="9" t="s">
         <v>40</v>
       </c>
-      <c r="I16" s="10">
+      <c r="J16" s="10">
         <v>4388756</v>
       </c>
-      <c r="J16" s="10">
+      <c r="K16" s="10">
         <v>26780526</v>
       </c>
-      <c r="L16" s="9" t="s">
+      <c r="M16" s="9" t="s">
         <v>42</v>
       </c>
-      <c r="M16">
+      <c r="N16">
         <v>0.09</v>
       </c>
     </row>
-    <row r="17" spans="5:13" x14ac:dyDescent="0.3">
+    <row r="17" spans="5:14" x14ac:dyDescent="0.3">
       <c r="E17" s="9" t="s">
         <v>31</v>
       </c>
       <c r="F17" s="10">
         <v>28948432</v>
       </c>
-      <c r="H17" s="9" t="s">
+      <c r="G17" s="10">
+        <v>31491260</v>
+      </c>
+      <c r="H17" s="10"/>
+      <c r="I17" s="9" t="s">
         <v>32</v>
       </c>
-      <c r="I17" s="10">
+      <c r="J17" s="10">
         <v>25712811</v>
       </c>
-      <c r="J17" s="10">
+      <c r="K17" s="10">
         <v>34670817</v>
       </c>
-      <c r="L17" s="11" t="s">
+      <c r="M17" s="11" t="s">
         <v>42</v>
       </c>
-      <c r="M17">
+      <c r="N17">
         <v>0.09</v>
       </c>
     </row>
-    <row r="18" spans="5:13" x14ac:dyDescent="0.3">
+    <row r="18" spans="5:14" x14ac:dyDescent="0.3">
       <c r="E18" s="9" t="s">
         <v>45</v>
       </c>
       <c r="F18" s="10">
         <v>11856728</v>
       </c>
-      <c r="H18" s="9" t="s">
+      <c r="G18" s="10">
+        <v>13494734</v>
+      </c>
+      <c r="H18" s="10"/>
+      <c r="I18" s="9" t="s">
         <v>69</v>
       </c>
-      <c r="I18" s="10">
+      <c r="J18" s="10">
         <v>151726</v>
       </c>
-      <c r="J18" s="10">
+      <c r="K18" s="10">
         <v>455962</v>
       </c>
-      <c r="L18" s="9" t="s">
+      <c r="M18" s="9" t="s">
         <v>43</v>
       </c>
-      <c r="M18">
+      <c r="N18">
         <v>2.11</v>
       </c>
     </row>
-    <row r="19" spans="5:13" x14ac:dyDescent="0.3">
+    <row r="19" spans="5:14" x14ac:dyDescent="0.3">
       <c r="E19" s="9" t="s">
         <v>50</v>
       </c>
       <c r="F19" s="10">
         <v>3382729</v>
       </c>
-      <c r="H19" s="9" t="s">
+      <c r="G19" s="10">
+        <v>3481873</v>
+      </c>
+      <c r="H19" s="10"/>
+      <c r="I19" s="9" t="s">
         <v>22</v>
       </c>
-      <c r="I19" s="10">
+      <c r="J19" s="10">
         <v>28219075</v>
       </c>
-      <c r="J19" s="10">
+      <c r="K19" s="10">
         <v>56361702</v>
       </c>
-      <c r="L19" s="11" t="s">
+      <c r="M19" s="11" t="s">
         <v>44</v>
       </c>
-      <c r="M19">
+      <c r="N19">
         <v>2.11</v>
       </c>
     </row>
-    <row r="20" spans="5:13" x14ac:dyDescent="0.3">
+    <row r="20" spans="5:14" x14ac:dyDescent="0.3">
       <c r="E20" s="9" t="s">
         <v>47</v>
       </c>
       <c r="F20" s="10">
         <v>5900640</v>
       </c>
-      <c r="H20" s="9" t="s">
+      <c r="G20" s="10">
+        <v>6640662</v>
+      </c>
+      <c r="H20" s="10"/>
+      <c r="I20" s="9" t="s">
         <v>57</v>
       </c>
-      <c r="I20" s="10">
+      <c r="J20" s="10">
         <v>822132</v>
       </c>
-      <c r="J20" s="10">
+      <c r="K20" s="10">
         <v>1899624</v>
       </c>
-      <c r="L20" s="9" t="s">
+      <c r="M20" s="9" t="s">
         <v>72</v>
       </c>
-      <c r="M20">
+      <c r="N20">
         <v>0.03</v>
       </c>
     </row>
-    <row r="21" spans="5:13" x14ac:dyDescent="0.3">
+    <row r="21" spans="5:14" x14ac:dyDescent="0.3">
       <c r="E21" s="9" t="s">
         <v>37</v>
       </c>
       <c r="F21" s="10">
         <v>16057819</v>
       </c>
-      <c r="H21" s="9" t="s">
+      <c r="G21" s="10">
+        <v>16930315</v>
+      </c>
+      <c r="H21" s="10"/>
+      <c r="I21" s="9" t="s">
         <v>63</v>
       </c>
-      <c r="I21" s="10">
+      <c r="J21" s="10">
         <v>313446</v>
       </c>
-      <c r="J21" s="10">
+      <c r="K21" s="10">
         <v>1069165</v>
       </c>
-      <c r="L21" s="11" t="s">
+      <c r="M21" s="11" t="s">
         <v>73</v>
       </c>
-      <c r="M21">
+      <c r="N21">
         <v>0.03</v>
       </c>
     </row>
-    <row r="22" spans="5:13" x14ac:dyDescent="0.3">
+    <row r="22" spans="5:14" x14ac:dyDescent="0.3">
       <c r="E22" s="9" t="s">
         <v>29</v>
       </c>
       <c r="F22" s="10">
         <v>30128640</v>
       </c>
-      <c r="H22" s="9" t="s">
+      <c r="G22" s="10">
+        <v>30966657</v>
+      </c>
+      <c r="H22" s="10"/>
+      <c r="I22" s="9" t="s">
         <v>28</v>
       </c>
-      <c r="I22" s="10">
+      <c r="J22" s="10">
         <v>17080776</v>
       </c>
-      <c r="J22" s="10">
+      <c r="K22" s="10">
         <v>51540236</v>
       </c>
-      <c r="L22" s="9" t="s">
+      <c r="M22" s="9" t="s">
         <v>74</v>
       </c>
-      <c r="M22">
+      <c r="N22">
         <v>0.02</v>
       </c>
     </row>
-    <row r="23" spans="5:13" x14ac:dyDescent="0.3">
+    <row r="23" spans="5:14" x14ac:dyDescent="0.3">
       <c r="E23" s="9" t="s">
         <v>35</v>
       </c>
       <c r="F23" s="10">
         <v>17378649</v>
       </c>
-      <c r="H23" s="9" t="s">
+      <c r="G23" s="10">
+        <v>16027412</v>
+      </c>
+      <c r="H23" s="10"/>
+      <c r="I23" s="9" t="s">
         <v>47</v>
       </c>
-      <c r="I23" s="10">
+      <c r="J23" s="10">
         <v>3414106</v>
       </c>
-      <c r="J23" s="10">
+      <c r="K23" s="10">
         <v>9134820</v>
       </c>
-      <c r="L23" s="11" t="s">
+      <c r="M23" s="11" t="s">
         <v>75</v>
       </c>
-      <c r="M23">
+      <c r="N23">
         <v>0.02</v>
       </c>
     </row>
-    <row r="24" spans="5:13" x14ac:dyDescent="0.3">
+    <row r="24" spans="5:14" x14ac:dyDescent="0.3">
       <c r="E24" s="9" t="s">
         <v>76</v>
       </c>
       <c r="F24" s="10">
         <v>31350</v>
       </c>
-      <c r="H24" s="9" t="s">
+      <c r="G24" s="10">
+        <v>33123</v>
+      </c>
+      <c r="H24" s="10"/>
+      <c r="I24" s="9" t="s">
         <v>77</v>
       </c>
-      <c r="I24" s="10">
+      <c r="J24" s="10">
         <v>50308</v>
       </c>
-      <c r="J24" s="10">
+      <c r="K24" s="10">
         <v>14121</v>
       </c>
-      <c r="L24" s="9" t="s">
+      <c r="M24" s="9" t="s">
         <v>46</v>
       </c>
-      <c r="M24">
+      <c r="N24">
         <v>1.39</v>
       </c>
     </row>
-    <row r="25" spans="5:13" x14ac:dyDescent="0.3">
+    <row r="25" spans="5:14" x14ac:dyDescent="0.3">
       <c r="E25" s="9" t="s">
         <v>23</v>
       </c>
       <c r="F25" s="10">
         <v>35014503</v>
       </c>
-      <c r="H25" s="9" t="s">
+      <c r="G25" s="10">
+        <v>37612306</v>
+      </c>
+      <c r="H25" s="10"/>
+      <c r="I25" s="9" t="s">
         <v>59</v>
       </c>
-      <c r="I25" s="10">
+      <c r="J25" s="10">
         <v>573741</v>
       </c>
-      <c r="J25" s="10">
+      <c r="K25" s="10">
         <v>1406861</v>
       </c>
-      <c r="L25" s="11" t="s">
+      <c r="M25" s="11" t="s">
         <v>46</v>
       </c>
-      <c r="M25">
+      <c r="N25">
         <v>1.39</v>
       </c>
     </row>
-    <row r="26" spans="5:13" x14ac:dyDescent="0.3">
+    <row r="26" spans="5:14" x14ac:dyDescent="0.3">
       <c r="E26" s="9" t="s">
         <v>15</v>
       </c>
       <c r="F26" s="10">
         <v>54131277</v>
       </c>
-      <c r="H26" s="9" t="s">
+      <c r="G26" s="10">
+        <v>58243056</v>
+      </c>
+      <c r="H26" s="10"/>
+      <c r="I26" s="9" t="s">
         <v>20</v>
       </c>
-      <c r="I26" s="10">
+      <c r="J26" s="10">
         <v>29134060</v>
       </c>
-      <c r="J26" s="10">
+      <c r="K26" s="10">
         <v>62213676</v>
       </c>
-      <c r="L26" s="9" t="s">
+      <c r="M26" s="9" t="s">
         <v>60</v>
       </c>
-      <c r="M26">
+      <c r="N26">
         <v>0.12</v>
       </c>
     </row>
-    <row r="27" spans="5:13" x14ac:dyDescent="0.3">
+    <row r="27" spans="5:14" x14ac:dyDescent="0.3">
       <c r="E27" s="9" t="s">
         <v>56</v>
       </c>
       <c r="F27" s="10">
         <v>1280219</v>
       </c>
-      <c r="H27" s="9" t="s">
+      <c r="G27" s="10">
+        <v>1290171</v>
+      </c>
+      <c r="H27" s="10"/>
+      <c r="I27" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="I27" s="10">
+      <c r="J27" s="10">
         <v>44470455</v>
       </c>
-      <c r="J27" s="10">
+      <c r="K27" s="10">
         <v>155111022</v>
       </c>
-      <c r="L27" s="11" t="s">
+      <c r="M27" s="11" t="s">
         <v>61</v>
       </c>
-      <c r="M27">
+      <c r="N27">
         <v>0.12</v>
       </c>
     </row>
-    <row r="28" spans="5:13" x14ac:dyDescent="0.3">
+    <row r="28" spans="5:14" x14ac:dyDescent="0.3">
       <c r="E28" s="9" t="s">
         <v>54</v>
       </c>
       <c r="F28" s="10">
         <v>1475057</v>
       </c>
-      <c r="H28" s="9" t="s">
+      <c r="G28" s="10">
+        <v>1491832</v>
+      </c>
+      <c r="H28" s="10"/>
+      <c r="I28" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="I28" s="10">
+      <c r="J28" s="10">
         <v>50827531</v>
       </c>
-      <c r="J28" s="10">
+      <c r="K28" s="10">
         <v>61545441</v>
       </c>
-      <c r="L28" s="9" t="s">
+      <c r="M28" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="M28">
+      <c r="N28">
         <v>4.99</v>
       </c>
     </row>
-    <row r="29" spans="5:13" x14ac:dyDescent="0.3">
+    <row r="29" spans="5:14" x14ac:dyDescent="0.3">
       <c r="E29" s="9" t="s">
         <v>66</v>
       </c>
       <c r="F29" s="10">
         <v>541867</v>
       </c>
-      <c r="H29" s="9" t="s">
+      <c r="G29" s="10">
+        <v>555339</v>
+      </c>
+      <c r="H29" s="10"/>
+      <c r="I29" s="9" t="s">
         <v>61</v>
       </c>
-      <c r="I29" s="10">
+      <c r="J29" s="10">
         <v>906309</v>
       </c>
-      <c r="J29" s="10">
+      <c r="K29" s="10">
         <v>551414</v>
       </c>
-      <c r="L29" s="11" t="s">
+      <c r="M29" s="11" t="s">
         <v>32</v>
       </c>
-      <c r="M29">
+      <c r="N29">
         <v>4.99</v>
       </c>
     </row>
-    <row r="30" spans="5:13" x14ac:dyDescent="0.3">
+    <row r="30" spans="5:14" x14ac:dyDescent="0.3">
       <c r="E30" s="9" t="s">
         <v>58</v>
       </c>
       <c r="F30" s="10">
         <v>953853</v>
       </c>
-      <c r="H30" s="9" t="s">
+      <c r="G30" s="10">
+        <v>1024649</v>
+      </c>
+      <c r="H30" s="10"/>
+      <c r="I30" s="9" t="s">
         <v>18</v>
       </c>
-      <c r="I30" s="10">
+      <c r="J30" s="10">
         <v>11729609</v>
       </c>
-      <c r="J30" s="10">
+      <c r="K30" s="10">
         <v>92075028</v>
       </c>
-      <c r="L30" s="9" t="s">
+      <c r="M30" s="9" t="s">
         <v>45</v>
       </c>
-      <c r="M30">
+      <c r="N30">
         <v>2.09</v>
       </c>
     </row>
-    <row r="31" spans="5:13" x14ac:dyDescent="0.3">
+    <row r="31" spans="5:14" x14ac:dyDescent="0.3">
       <c r="E31" s="9" t="s">
         <v>33</v>
       </c>
       <c r="F31" s="10">
         <v>20762082</v>
       </c>
-      <c r="H31" s="9" t="s">
+      <c r="G31" s="10">
+        <v>21212136</v>
+      </c>
+      <c r="H31" s="10"/>
+      <c r="I31" s="9" t="s">
         <v>65</v>
       </c>
-      <c r="I31" s="10">
+      <c r="J31" s="10">
         <v>850123</v>
       </c>
-      <c r="J31" s="10">
+      <c r="K31" s="10">
         <v>394341</v>
       </c>
-      <c r="L31" s="11" t="s">
+      <c r="M31" s="11" t="s">
         <v>42</v>
       </c>
-      <c r="M31">
+      <c r="N31">
         <v>2.09</v>
       </c>
     </row>
-    <row r="32" spans="5:13" x14ac:dyDescent="0.3">
+    <row r="32" spans="5:14" x14ac:dyDescent="0.3">
       <c r="E32" s="9" t="s">
         <v>64</v>
       </c>
       <c r="F32" s="10">
         <v>635442</v>
       </c>
-      <c r="H32" s="9" t="s">
+      <c r="G32" s="10">
+        <v>612511</v>
+      </c>
+      <c r="H32" s="10"/>
+      <c r="I32" s="9" t="s">
         <v>71</v>
       </c>
-      <c r="I32" s="10">
+      <c r="J32" s="10">
         <v>135533</v>
       </c>
-      <c r="J32" s="10">
+      <c r="K32" s="10">
         <v>244411</v>
       </c>
-      <c r="L32" s="9" t="s">
+      <c r="M32" s="9" t="s">
         <v>50</v>
       </c>
-      <c r="M32">
+      <c r="N32">
         <v>0.56999999999999995</v>
       </c>
     </row>
-    <row r="33" spans="5:13" x14ac:dyDescent="0.3">
+    <row r="33" spans="5:14" x14ac:dyDescent="0.3">
       <c r="E33" s="9" t="s">
         <v>41</v>
       </c>
       <c r="F33" s="10">
         <v>13103873</v>
       </c>
-      <c r="H33" s="9" t="s">
+      <c r="G33" s="10">
+        <v>14639465</v>
+      </c>
+      <c r="H33" s="10"/>
+      <c r="I33" s="9" t="s">
         <v>44</v>
       </c>
-      <c r="I33" s="10">
+      <c r="J33" s="10">
         <v>5936538</v>
       </c>
-      <c r="J33" s="10">
+      <c r="K33" s="10">
         <v>19603658</v>
       </c>
-      <c r="L33" s="11" t="s">
+      <c r="M33" s="11" t="s">
         <v>51</v>
       </c>
-      <c r="M33">
+      <c r="N33">
         <v>0.56999999999999995</v>
       </c>
     </row>
-    <row r="34" spans="5:13" x14ac:dyDescent="0.3">
+    <row r="34" spans="5:14" x14ac:dyDescent="0.3">
       <c r="E34" s="9" t="s">
         <v>27</v>
       </c>
       <c r="F34" s="10">
         <v>32997440</v>
       </c>
-      <c r="H34" s="9" t="s">
+      <c r="G34" s="10">
+        <v>35550997</v>
+      </c>
+      <c r="H34" s="10"/>
+      <c r="I34" s="9" t="s">
         <v>38</v>
       </c>
-      <c r="I34" s="10">
+      <c r="J34" s="10">
         <v>7929292</v>
       </c>
-      <c r="J34" s="10">
+      <c r="K34" s="10">
         <v>25036946</v>
       </c>
-      <c r="L34" s="9" t="s">
+      <c r="M34" s="9" t="s">
         <v>47</v>
       </c>
-      <c r="M34">
+      <c r="N34">
         <v>1.04</v>
       </c>
     </row>
-    <row r="35" spans="5:13" x14ac:dyDescent="0.3">
+    <row r="35" spans="5:14" x14ac:dyDescent="0.3">
       <c r="E35" s="9" t="s">
         <v>68</v>
       </c>
       <c r="F35" s="10">
         <v>287507</v>
       </c>
-      <c r="H35" s="9" t="s">
+      <c r="G35" s="10">
+        <v>323070</v>
+      </c>
+      <c r="H35" s="10"/>
+      <c r="I35" s="9" t="s">
         <v>55</v>
       </c>
-      <c r="I35" s="10">
+      <c r="J35" s="10">
         <v>595036</v>
       </c>
-      <c r="J35" s="10">
+      <c r="K35" s="10">
         <v>2368971</v>
       </c>
-      <c r="L35" s="11" t="s">
+      <c r="M35" s="11" t="s">
         <v>47</v>
       </c>
-      <c r="M35">
+      <c r="N35">
         <v>1.04</v>
       </c>
     </row>
-    <row r="36" spans="5:13" x14ac:dyDescent="0.3">
+    <row r="36" spans="5:14" x14ac:dyDescent="0.3">
       <c r="E36" s="9" t="s">
         <v>25</v>
       </c>
       <c r="F36" s="10">
         <v>36009055</v>
       </c>
-      <c r="H36" s="9" t="s">
+      <c r="G36" s="10">
+        <v>36137975</v>
+      </c>
+      <c r="H36" s="10"/>
+      <c r="I36" s="9" t="s">
         <v>51</v>
       </c>
-      <c r="I36" s="10">
+      <c r="J36" s="10">
         <v>688704</v>
       </c>
-      <c r="J36" s="10">
+      <c r="K36" s="10">
         <v>6167805</v>
       </c>
-      <c r="L36" s="9" t="s">
+      <c r="M36" s="9" t="s">
         <v>37</v>
       </c>
-      <c r="M36">
+      <c r="N36">
         <v>2.72</v>
       </c>
     </row>
-    <row r="37" spans="5:13" x14ac:dyDescent="0.3">
+    <row r="37" spans="5:14" x14ac:dyDescent="0.3">
       <c r="E37" s="9" t="s">
         <v>52</v>
       </c>
       <c r="F37" s="10">
         <v>1799541</v>
       </c>
-      <c r="H37" s="9" t="s">
+      <c r="G37" s="10">
+        <v>1874376</v>
+      </c>
+      <c r="H37" s="10"/>
+      <c r="I37" s="9" t="s">
         <v>73</v>
       </c>
-      <c r="I37" s="10">
+      <c r="J37" s="10">
         <v>159829</v>
       </c>
-      <c r="J37" s="10">
+      <c r="K37" s="10">
         <v>183024</v>
       </c>
-      <c r="L37" s="11" t="s">
+      <c r="M37" s="11" t="s">
         <v>38</v>
       </c>
-      <c r="M37">
+      <c r="N37">
         <v>2.72</v>
       </c>
     </row>
-    <row r="38" spans="5:13" x14ac:dyDescent="0.3">
+    <row r="38" spans="5:14" x14ac:dyDescent="0.3">
       <c r="E38" s="9" t="s">
         <v>13</v>
       </c>
       <c r="F38" s="10">
         <v>95331831</v>
       </c>
-      <c r="H38" s="9" t="s">
+      <c r="G38" s="10">
+        <v>104480510</v>
+      </c>
+      <c r="H38" s="10"/>
+      <c r="I38" s="9" t="s">
         <v>36</v>
       </c>
-      <c r="I38" s="10">
+      <c r="J38" s="10">
         <v>15932171</v>
       </c>
-      <c r="J38" s="10">
+      <c r="K38" s="10">
         <v>17445506</v>
       </c>
-      <c r="L38" s="9" t="s">
+      <c r="M38" s="9" t="s">
         <v>29</v>
       </c>
-      <c r="M38">
+      <c r="N38">
         <v>5.05</v>
       </c>
     </row>
-    <row r="39" spans="5:13" x14ac:dyDescent="0.3">
+    <row r="39" spans="5:14" x14ac:dyDescent="0.3">
       <c r="E39" s="9" t="s">
         <v>48</v>
       </c>
       <c r="F39" s="10">
         <v>4948519</v>
       </c>
-      <c r="H39" s="9" t="s">
+      <c r="G39" s="10">
+        <v>5137773</v>
+      </c>
+      <c r="H39" s="10"/>
+      <c r="I39" s="9" t="s">
         <v>89</v>
       </c>
-      <c r="I39" s="10">
+      <c r="J39" s="10">
         <v>373542974</v>
       </c>
-      <c r="J39" s="10">
+      <c r="K39" s="10">
         <v>833652994</v>
       </c>
-      <c r="L39" s="11" t="s">
+      <c r="M39" s="11" t="s">
         <v>30</v>
       </c>
-      <c r="M39">
+      <c r="N39">
         <v>5.05</v>
       </c>
     </row>
-    <row r="40" spans="5:13" x14ac:dyDescent="0.3">
+    <row r="40" spans="5:14" x14ac:dyDescent="0.3">
       <c r="E40" s="9" t="s">
         <v>19</v>
       </c>
       <c r="F40" s="10">
         <v>44467088</v>
       </c>
-      <c r="L40" s="9" t="s">
+      <c r="G40" s="10">
+        <v>46809027</v>
+      </c>
+      <c r="H40" s="10"/>
+      <c r="M40" s="9" t="s">
         <v>35</v>
       </c>
-      <c r="M40">
+      <c r="N40">
         <v>2.76</v>
       </c>
     </row>
-    <row r="41" spans="5:13" x14ac:dyDescent="0.3">
+    <row r="41" spans="5:14" x14ac:dyDescent="0.3">
       <c r="E41" s="9" t="s">
         <v>89</v>
       </c>
       <c r="F41" s="10">
         <v>587447730</v>
       </c>
-      <c r="L41" s="11" t="s">
+      <c r="G41" s="10">
+        <v>623021843</v>
+      </c>
+      <c r="H41" s="10"/>
+      <c r="M41" s="11" t="s">
         <v>36</v>
       </c>
-      <c r="M41">
+      <c r="N41">
         <v>2.76</v>
       </c>
     </row>
-    <row r="42" spans="5:13" x14ac:dyDescent="0.3">
-      <c r="L42" s="9" t="s">
+    <row r="42" spans="5:14" x14ac:dyDescent="0.3">
+      <c r="M42" s="9" t="s">
         <v>76</v>
       </c>
-      <c r="M42">
+      <c r="N42">
         <v>0.01</v>
       </c>
     </row>
-    <row r="43" spans="5:13" x14ac:dyDescent="0.3">
-      <c r="L43" s="11" t="s">
+    <row r="43" spans="5:14" x14ac:dyDescent="0.3">
+      <c r="M43" s="11" t="s">
         <v>77</v>
       </c>
-      <c r="M43">
+      <c r="N43">
         <v>0.01</v>
       </c>
     </row>
-    <row r="44" spans="5:13" x14ac:dyDescent="0.3">
-      <c r="L44" s="9" t="s">
+    <row r="44" spans="5:14" x14ac:dyDescent="0.3">
+      <c r="M44" s="9" t="s">
         <v>23</v>
       </c>
-      <c r="M44">
+      <c r="N44">
         <v>6</v>
       </c>
     </row>
-    <row r="45" spans="5:13" x14ac:dyDescent="0.3">
-      <c r="L45" s="11" t="s">
+    <row r="45" spans="5:14" x14ac:dyDescent="0.3">
+      <c r="M45" s="11" t="s">
         <v>24</v>
       </c>
-      <c r="M45">
+      <c r="N45">
         <v>6</v>
       </c>
     </row>
-    <row r="46" spans="5:13" x14ac:dyDescent="0.3">
-      <c r="L46" s="9" t="s">
+    <row r="46" spans="5:14" x14ac:dyDescent="0.3">
+      <c r="M46" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="M46">
+      <c r="N46">
         <v>9.2799999999999994</v>
       </c>
     </row>
-    <row r="47" spans="5:13" x14ac:dyDescent="0.3">
-      <c r="L47" s="11" t="s">
+    <row r="47" spans="5:14" x14ac:dyDescent="0.3">
+      <c r="M47" s="11" t="s">
         <v>16</v>
       </c>
-      <c r="M47">
+      <c r="N47">
         <v>9.2799999999999994</v>
       </c>
     </row>
-    <row r="48" spans="5:13" x14ac:dyDescent="0.3">
-      <c r="L48" s="9" t="s">
+    <row r="48" spans="5:14" x14ac:dyDescent="0.3">
+      <c r="M48" s="9" t="s">
         <v>56</v>
       </c>
-      <c r="M48">
+      <c r="N48">
         <v>0.21</v>
       </c>
     </row>
-    <row r="49" spans="12:13" x14ac:dyDescent="0.3">
-      <c r="L49" s="11" t="s">
+    <row r="49" spans="13:14" x14ac:dyDescent="0.3">
+      <c r="M49" s="11" t="s">
         <v>57</v>
       </c>
-      <c r="M49">
+      <c r="N49">
         <v>0.21</v>
       </c>
     </row>
-    <row r="50" spans="12:13" x14ac:dyDescent="0.3">
-      <c r="L50" s="9" t="s">
+    <row r="50" spans="13:14" x14ac:dyDescent="0.3">
+      <c r="M50" s="9" t="s">
         <v>54</v>
       </c>
-      <c r="M50">
+      <c r="N50">
         <v>0.25</v>
       </c>
     </row>
-    <row r="51" spans="12:13" x14ac:dyDescent="0.3">
-      <c r="L51" s="11" t="s">
+    <row r="51" spans="13:14" x14ac:dyDescent="0.3">
+      <c r="M51" s="11" t="s">
         <v>55</v>
       </c>
-      <c r="M51">
+      <c r="N51">
         <v>0.25</v>
       </c>
     </row>
-    <row r="52" spans="12:13" x14ac:dyDescent="0.3">
-      <c r="L52" s="9" t="s">
+    <row r="52" spans="13:14" x14ac:dyDescent="0.3">
+      <c r="M52" s="9" t="s">
         <v>66</v>
       </c>
-      <c r="M52">
+      <c r="N52">
         <v>0.09</v>
       </c>
     </row>
-    <row r="53" spans="12:13" x14ac:dyDescent="0.3">
-      <c r="L53" s="11" t="s">
+    <row r="53" spans="13:14" x14ac:dyDescent="0.3">
+      <c r="M53" s="11" t="s">
         <v>67</v>
       </c>
-      <c r="M53">
+      <c r="N53">
         <v>0.09</v>
       </c>
     </row>
-    <row r="54" spans="12:13" x14ac:dyDescent="0.3">
-      <c r="L54" s="9" t="s">
+    <row r="54" spans="13:14" x14ac:dyDescent="0.3">
+      <c r="M54" s="9" t="s">
         <v>58</v>
       </c>
-      <c r="M54">
+      <c r="N54">
         <v>0.16</v>
       </c>
     </row>
-    <row r="55" spans="12:13" x14ac:dyDescent="0.3">
-      <c r="L55" s="11" t="s">
+    <row r="55" spans="13:14" x14ac:dyDescent="0.3">
+      <c r="M55" s="11" t="s">
         <v>59</v>
       </c>
-      <c r="M55">
+      <c r="N55">
         <v>0.16</v>
       </c>
     </row>
-    <row r="56" spans="12:13" x14ac:dyDescent="0.3">
-      <c r="L56" s="9" t="s">
+    <row r="56" spans="13:14" x14ac:dyDescent="0.3">
+      <c r="M56" s="9" t="s">
         <v>33</v>
       </c>
-      <c r="M56">
+      <c r="N56">
         <v>3.47</v>
       </c>
     </row>
-    <row r="57" spans="12:13" x14ac:dyDescent="0.3">
-      <c r="L57" s="11" t="s">
+    <row r="57" spans="13:14" x14ac:dyDescent="0.3">
+      <c r="M57" s="11" t="s">
         <v>34</v>
       </c>
-      <c r="M57">
+      <c r="N57">
         <v>3.47</v>
       </c>
     </row>
-    <row r="58" spans="12:13" x14ac:dyDescent="0.3">
-      <c r="L58" s="9" t="s">
+    <row r="58" spans="13:14" x14ac:dyDescent="0.3">
+      <c r="M58" s="9" t="s">
         <v>64</v>
       </c>
-      <c r="M58">
+      <c r="N58">
         <v>0.1</v>
       </c>
     </row>
-    <row r="59" spans="12:13" x14ac:dyDescent="0.3">
-      <c r="L59" s="11" t="s">
+    <row r="59" spans="13:14" x14ac:dyDescent="0.3">
+      <c r="M59" s="11" t="s">
         <v>65</v>
       </c>
-      <c r="M59">
+      <c r="N59">
         <v>0.1</v>
       </c>
     </row>
-    <row r="60" spans="12:13" x14ac:dyDescent="0.3">
-      <c r="L60" s="9" t="s">
+    <row r="60" spans="13:14" x14ac:dyDescent="0.3">
+      <c r="M60" s="9" t="s">
         <v>41</v>
       </c>
-      <c r="M60">
+      <c r="N60">
         <v>2.29</v>
       </c>
     </row>
-    <row r="61" spans="12:13" x14ac:dyDescent="0.3">
-      <c r="L61" s="11" t="s">
+    <row r="61" spans="13:14" x14ac:dyDescent="0.3">
+      <c r="M61" s="11" t="s">
         <v>42</v>
       </c>
-      <c r="M61">
+      <c r="N61">
         <v>2.29</v>
       </c>
     </row>
-    <row r="62" spans="12:13" x14ac:dyDescent="0.3">
-      <c r="L62" s="9" t="s">
+    <row r="62" spans="13:14" x14ac:dyDescent="0.3">
+      <c r="M62" s="9" t="s">
         <v>27</v>
       </c>
-      <c r="M62">
+      <c r="N62">
         <v>5.66</v>
       </c>
     </row>
-    <row r="63" spans="12:13" x14ac:dyDescent="0.3">
-      <c r="L63" s="11" t="s">
+    <row r="63" spans="13:14" x14ac:dyDescent="0.3">
+      <c r="M63" s="11" t="s">
         <v>28</v>
       </c>
-      <c r="M63">
+      <c r="N63">
         <v>5.66</v>
       </c>
     </row>
-    <row r="64" spans="12:13" x14ac:dyDescent="0.3">
-      <c r="L64" s="9" t="s">
+    <row r="64" spans="13:14" x14ac:dyDescent="0.3">
+      <c r="M64" s="9" t="s">
         <v>68</v>
       </c>
-      <c r="M64">
+      <c r="N64">
         <v>0.05</v>
       </c>
     </row>
-    <row r="65" spans="12:13" x14ac:dyDescent="0.3">
-      <c r="L65" s="11" t="s">
+    <row r="65" spans="13:14" x14ac:dyDescent="0.3">
+      <c r="M65" s="11" t="s">
         <v>69</v>
       </c>
-      <c r="M65">
+      <c r="N65">
         <v>0.05</v>
       </c>
     </row>
-    <row r="66" spans="12:13" x14ac:dyDescent="0.3">
-      <c r="L66" s="9" t="s">
+    <row r="66" spans="13:14" x14ac:dyDescent="0.3">
+      <c r="M66" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="M66">
+      <c r="N66">
         <v>5.96</v>
       </c>
     </row>
-    <row r="67" spans="12:13" x14ac:dyDescent="0.3">
-      <c r="L67" s="11" t="s">
+    <row r="67" spans="13:14" x14ac:dyDescent="0.3">
+      <c r="M67" s="11" t="s">
         <v>26</v>
       </c>
-      <c r="M67">
+      <c r="N67">
         <v>5.96</v>
       </c>
     </row>
-    <row r="68" spans="12:13" x14ac:dyDescent="0.3">
-      <c r="L68" s="9" t="s">
+    <row r="68" spans="13:14" x14ac:dyDescent="0.3">
+      <c r="M68" s="9" t="s">
         <v>52</v>
       </c>
-      <c r="M68">
+      <c r="N68">
         <v>0.3</v>
       </c>
     </row>
-    <row r="69" spans="12:13" x14ac:dyDescent="0.3">
-      <c r="L69" s="11" t="s">
+    <row r="69" spans="13:14" x14ac:dyDescent="0.3">
+      <c r="M69" s="11" t="s">
         <v>53</v>
       </c>
-      <c r="M69">
+      <c r="N69">
         <v>0.3</v>
       </c>
     </row>
-    <row r="70" spans="12:13" x14ac:dyDescent="0.3">
-      <c r="L70" s="9" t="s">
+    <row r="70" spans="13:14" x14ac:dyDescent="0.3">
+      <c r="M70" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="M70">
+      <c r="N70">
         <v>16.5</v>
       </c>
     </row>
-    <row r="71" spans="12:13" x14ac:dyDescent="0.3">
-      <c r="L71" s="11" t="s">
+    <row r="71" spans="13:14" x14ac:dyDescent="0.3">
+      <c r="M71" s="11" t="s">
         <v>14</v>
       </c>
-      <c r="M71">
+      <c r="N71">
         <v>16.5</v>
       </c>
     </row>
-    <row r="72" spans="12:13" x14ac:dyDescent="0.3">
-      <c r="L72" s="9" t="s">
+    <row r="72" spans="13:14" x14ac:dyDescent="0.3">
+      <c r="M72" s="9" t="s">
         <v>48</v>
       </c>
-      <c r="M72">
+      <c r="N72">
         <v>0.83</v>
       </c>
     </row>
-    <row r="73" spans="12:13" x14ac:dyDescent="0.3">
-      <c r="L73" s="11" t="s">
+    <row r="73" spans="13:14" x14ac:dyDescent="0.3">
+      <c r="M73" s="11" t="s">
         <v>49</v>
       </c>
-      <c r="M73">
+      <c r="N73">
         <v>0.83</v>
       </c>
     </row>
-    <row r="74" spans="12:13" x14ac:dyDescent="0.3">
-      <c r="L74" s="9" t="s">
+    <row r="74" spans="13:14" x14ac:dyDescent="0.3">
+      <c r="M74" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="M74">
+      <c r="N74">
         <v>7.54</v>
       </c>
     </row>
-    <row r="75" spans="12:13" x14ac:dyDescent="0.3">
-      <c r="L75" s="11" t="s">
+    <row r="75" spans="13:14" x14ac:dyDescent="0.3">
+      <c r="M75" s="11" t="s">
         <v>20</v>
       </c>
-      <c r="M75">
+      <c r="N75">
         <v>7.54</v>
       </c>
     </row>
-    <row r="76" spans="12:13" x14ac:dyDescent="0.3">
-      <c r="L76" s="9" t="s">
+    <row r="76" spans="13:14" x14ac:dyDescent="0.3">
+      <c r="M76" s="9" t="s">
         <v>89</v>
       </c>
-      <c r="M76">
+      <c r="N76">
         <v>99.99</v>
       </c>
     </row>

</xml_diff>